<commit_message>
add code for 3d data
</commit_message>
<xml_diff>
--- a/dataset_test-v2.xlsx
+++ b/dataset_test-v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\qiqilu\Project\2024 Foundation model\code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30B8E7FD-38BE-4F87-9E8E-2154716AA828}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3CEFB0F-E701-4A7B-BDED-4CAD5DFF5589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1515" yWindow="1515" windowWidth="29715" windowHeight="17190" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18540" yWindow="2520" windowWidth="16785" windowHeight="17190" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10108" uniqueCount="1574">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10123" uniqueCount="1579">
   <si>
     <t>path_lr</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -5575,6 +5575,26 @@
   </si>
   <si>
     <t>FMD-2photon-BPAE-r-2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3dsim-fixedga-ltdr-gal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3DSIM-FixedGA-GAL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3dsim-fixed-pfa-egfp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3DSIM-PFA</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fixed rat cardiomyoblast cell-line H9c2</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -8822,7 +8842,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58090EBB-A764-4E1D-A677-EA141CD033B7}">
-  <dimension ref="A1:AC452"/>
+  <dimension ref="A1:AC456"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -48473,6 +48493,88 @@
       </c>
       <c r="AC452" s="32" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="453" spans="1:29" s="67" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A453" s="67">
+        <v>40001</v>
+      </c>
+      <c r="B453" s="67" t="s">
+        <v>1574</v>
+      </c>
+      <c r="C453" s="67" t="s">
+        <v>1575</v>
+      </c>
+      <c r="D453" s="67" t="s">
+        <v>1278</v>
+      </c>
+      <c r="E453" s="78" t="s">
+        <v>1201</v>
+      </c>
+      <c r="F453" s="78" t="s">
+        <v>1201</v>
+      </c>
+      <c r="G453" s="64">
+        <v>3</v>
+      </c>
+      <c r="R453" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="T453" s="68"/>
+      <c r="W453" s="68"/>
+      <c r="X453" s="64"/>
+      <c r="Y453" s="69"/>
+      <c r="AA453" s="68"/>
+      <c r="AB453" s="64"/>
+      <c r="AC453" s="69"/>
+    </row>
+    <row r="454" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A454" s="70">
+        <v>40002</v>
+      </c>
+    </row>
+    <row r="455" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A455" s="70"/>
+    </row>
+    <row r="456" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="B456" t="s">
+        <v>1576</v>
+      </c>
+      <c r="C456" t="s">
+        <v>1577</v>
+      </c>
+      <c r="D456" t="s">
+        <v>1278</v>
+      </c>
+      <c r="E456" s="2" t="s">
+        <v>1201</v>
+      </c>
+      <c r="F456" s="2" t="s">
+        <v>1201</v>
+      </c>
+      <c r="G456" s="23">
+        <v>3</v>
+      </c>
+      <c r="H456" s="70" t="s">
+        <v>163</v>
+      </c>
+      <c r="I456" s="70" t="s">
+        <v>104</v>
+      </c>
+      <c r="J456">
+        <v>2</v>
+      </c>
+      <c r="K456">
+        <v>1</v>
+      </c>
+      <c r="M456">
+        <v>8</v>
+      </c>
+      <c r="R456" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="S456" t="s">
+        <v>1578</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add code for structural prompt
</commit_message>
<xml_diff>
--- a/dataset_test-v2.xlsx
+++ b/dataset_test-v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\qiqilu\Project\2024 Foundation model\code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B9AB71F-3C82-4C03-A13D-7DFA1BC282B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22DE3D4E-D0EA-4E43-94F0-377FCBE9B4F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1335" yWindow="2370" windowWidth="16785" windowHeight="17190" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18165" yWindow="2715" windowWidth="16785" windowHeight="17190" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11864" uniqueCount="1701">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11833" uniqueCount="1698">
   <si>
     <t>path_lr</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -6012,18 +6012,6 @@
   </si>
   <si>
     <t>E:\qiqilu\datasets\DL-SMLM\transformed\Microtubules\test.txt</t>
-  </si>
-  <si>
-    <t>rcan3d-c2s-mt-dcv-mc-3d</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>RCAN-C2S-MT-mc-3d</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>dcv-real3d</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -6348,54 +6336,7 @@
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="362">
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="357">
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -9519,7 +9460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58090EBB-A764-4E1D-A677-EA141CD033B7}">
-  <dimension ref="A1:AE497"/>
+  <dimension ref="A1:AE487"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -51933,16 +51874,49 @@
     </row>
     <row r="454" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A454" s="70">
-        <v>40002</v>
+        <v>40004</v>
+      </c>
+      <c r="B454" t="s">
+        <v>1576</v>
+      </c>
+      <c r="C454" t="s">
+        <v>1577</v>
+      </c>
+      <c r="D454" t="s">
+        <v>1278</v>
+      </c>
+      <c r="E454" s="2" t="s">
+        <v>1201</v>
+      </c>
+      <c r="F454" s="2" t="s">
+        <v>1201</v>
       </c>
       <c r="G454" s="23">
         <v>3</v>
       </c>
-      <c r="K454" s="4">
-        <v>-3</v>
+      <c r="H454" s="70" t="s">
+        <v>163</v>
+      </c>
+      <c r="I454" s="70" t="s">
+        <v>104</v>
+      </c>
+      <c r="J454">
+        <v>2</v>
+      </c>
+      <c r="K454">
+        <v>1</v>
+      </c>
+      <c r="M454">
+        <v>8</v>
       </c>
       <c r="P454" s="38" t="s">
         <v>572</v>
+      </c>
+      <c r="R454" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="S454" t="s">
+        <v>1578</v>
       </c>
       <c r="Z454" s="33" t="s">
         <v>1048</v>
@@ -51953,54 +51927,126 @@
     </row>
     <row r="455" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A455" s="70">
-        <v>40003</v>
+        <v>40005</v>
+      </c>
+      <c r="B455" s="63" t="s">
+        <v>1579</v>
+      </c>
+      <c r="C455" s="63" t="s">
+        <v>1580</v>
+      </c>
+      <c r="D455" s="73" t="s">
+        <v>1278</v>
+      </c>
+      <c r="E455" s="73" t="s">
+        <v>1201</v>
+      </c>
+      <c r="F455" s="73" t="s">
+        <v>1201</v>
       </c>
       <c r="G455" s="23">
         <v>3</v>
       </c>
-      <c r="K455" s="4">
-        <v>-3</v>
+      <c r="H455" s="71" t="s">
+        <v>111</v>
+      </c>
+      <c r="I455" s="73" t="s">
+        <v>105</v>
+      </c>
+      <c r="J455">
+        <v>1</v>
+      </c>
+      <c r="K455">
+        <v>1</v>
+      </c>
+      <c r="M455">
+        <v>8</v>
+      </c>
+      <c r="N455" t="s">
+        <v>1591</v>
+      </c>
+      <c r="O455" t="s">
+        <v>1592</v>
       </c>
       <c r="P455" s="38" t="s">
         <v>572</v>
       </c>
-      <c r="Z455" s="33" t="s">
-        <v>1048</v>
-      </c>
-      <c r="AE455" s="33" t="s">
-        <v>1048</v>
+      <c r="Q455" t="s">
+        <v>1586</v>
+      </c>
+      <c r="R455" s="33" t="s">
+        <v>95</v>
+      </c>
+      <c r="S455" s="62" t="s">
+        <v>784</v>
+      </c>
+      <c r="T455" s="83" t="s">
+        <v>964</v>
+      </c>
+      <c r="U455" s="67" t="s">
+        <v>1000</v>
+      </c>
+      <c r="V455" s="62" t="s">
+        <v>788</v>
+      </c>
+      <c r="W455" s="102" t="s">
+        <v>933</v>
+      </c>
+      <c r="X455" s="103" t="s">
+        <v>1038</v>
+      </c>
+      <c r="Y455" s="101" t="s">
+        <v>785</v>
+      </c>
+      <c r="Z455" s="101" t="s">
+        <v>1595</v>
+      </c>
+      <c r="AA455" s="62" t="s">
+        <v>787</v>
+      </c>
+      <c r="AB455" s="102" t="s">
+        <v>1011</v>
+      </c>
+      <c r="AC455" s="103" t="s">
+        <v>1038</v>
+      </c>
+      <c r="AD455" s="101" t="s">
+        <v>785</v>
+      </c>
+      <c r="AE455" s="101" t="s">
+        <v>1595</v>
       </c>
     </row>
     <row r="456" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A456" s="70">
-        <v>40004</v>
-      </c>
-      <c r="B456" t="s">
-        <v>1576</v>
-      </c>
-      <c r="C456" t="s">
-        <v>1577</v>
-      </c>
-      <c r="D456" t="s">
+        <v>40006</v>
+      </c>
+      <c r="B456" s="73" t="s">
+        <v>1581</v>
+      </c>
+      <c r="C456" s="73" t="s">
+        <v>1582</v>
+      </c>
+      <c r="D456" s="73" t="s">
         <v>1278</v>
       </c>
-      <c r="E456" s="2" t="s">
+      <c r="E456" s="73" t="s">
         <v>1201</v>
       </c>
-      <c r="F456" s="2" t="s">
+      <c r="F456" s="73" t="s">
         <v>1201</v>
       </c>
       <c r="G456" s="23">
         <v>3</v>
       </c>
-      <c r="H456" s="70" t="s">
-        <v>163</v>
-      </c>
-      <c r="I456" s="70" t="s">
-        <v>104</v>
+      <c r="H456" s="71" t="s">
+        <v>781</v>
+      </c>
+      <c r="I456" s="73" t="s">
+        <v>105</v>
       </c>
       <c r="J456">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K456">
         <v>1</v>
@@ -52008,31 +52054,70 @@
       <c r="M456">
         <v>8</v>
       </c>
+      <c r="N456" t="s">
+        <v>1593</v>
+      </c>
+      <c r="O456" t="s">
+        <v>1594</v>
+      </c>
       <c r="P456" s="38" t="s">
         <v>572</v>
       </c>
-      <c r="R456" s="31" t="s">
-        <v>11</v>
-      </c>
-      <c r="S456" t="s">
-        <v>1578</v>
+      <c r="Q456" t="s">
+        <v>1587</v>
+      </c>
+      <c r="R456" s="33" t="s">
+        <v>95</v>
+      </c>
+      <c r="S456" s="71" t="s">
+        <v>784</v>
+      </c>
+      <c r="T456" s="31" t="s">
+        <v>967</v>
+      </c>
+      <c r="U456" t="s">
+        <v>1001</v>
+      </c>
+      <c r="V456" s="71" t="s">
+        <v>789</v>
+      </c>
+      <c r="W456" s="28" t="s">
+        <v>933</v>
+      </c>
+      <c r="X456" s="20" t="s">
+        <v>1038</v>
+      </c>
+      <c r="Y456" s="33" t="s">
+        <v>786</v>
       </c>
       <c r="Z456" s="33" t="s">
-        <v>1048</v>
+        <v>1595</v>
+      </c>
+      <c r="AA456" s="71" t="s">
+        <v>787</v>
+      </c>
+      <c r="AB456" s="28" t="s">
+        <v>1011</v>
+      </c>
+      <c r="AC456" s="20" t="s">
+        <v>1038</v>
+      </c>
+      <c r="AD456" s="33" t="s">
+        <v>786</v>
       </c>
       <c r="AE456" s="33" t="s">
-        <v>1048</v>
+        <v>1595</v>
       </c>
     </row>
     <row r="457" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A457" s="70">
-        <v>40005</v>
-      </c>
-      <c r="B457" s="63" t="s">
-        <v>1579</v>
-      </c>
-      <c r="C457" s="63" t="s">
-        <v>1580</v>
+        <v>40007</v>
+      </c>
+      <c r="B457" s="73" t="s">
+        <v>1583</v>
+      </c>
+      <c r="C457" s="73" t="s">
+        <v>1584</v>
       </c>
       <c r="D457" s="73" t="s">
         <v>1278</v>
@@ -52047,7 +52132,7 @@
         <v>3</v>
       </c>
       <c r="H457" s="71" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="I457" s="73" t="s">
         <v>105</v>
@@ -52062,161 +52147,161 @@
         <v>8</v>
       </c>
       <c r="N457" t="s">
-        <v>1591</v>
+        <v>1589</v>
       </c>
       <c r="O457" t="s">
-        <v>1592</v>
+        <v>1590</v>
       </c>
       <c r="P457" s="38" t="s">
         <v>572</v>
       </c>
       <c r="Q457" t="s">
-        <v>1586</v>
+        <v>1588</v>
       </c>
       <c r="R457" s="33" t="s">
         <v>95</v>
       </c>
-      <c r="S457" s="62" t="s">
+      <c r="S457" s="71" t="s">
         <v>784</v>
       </c>
-      <c r="T457" s="83" t="s">
-        <v>964</v>
-      </c>
-      <c r="U457" s="67" t="s">
-        <v>1000</v>
-      </c>
-      <c r="V457" s="62" t="s">
-        <v>788</v>
-      </c>
-      <c r="W457" s="102" t="s">
+      <c r="T457" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="U457" s="71" t="s">
+        <v>1585</v>
+      </c>
+      <c r="V457" s="71" t="s">
+        <v>1201</v>
+      </c>
+      <c r="W457" s="28" t="s">
         <v>933</v>
       </c>
-      <c r="X457" s="103" t="s">
+      <c r="X457" s="20" t="s">
         <v>1038</v>
       </c>
-      <c r="Y457" s="101" t="s">
-        <v>785</v>
-      </c>
-      <c r="Z457" s="101" t="s">
+      <c r="Y457" s="33" t="s">
+        <v>786</v>
+      </c>
+      <c r="Z457" s="33" t="s">
         <v>1595</v>
       </c>
-      <c r="AA457" s="62" t="s">
-        <v>787</v>
-      </c>
-      <c r="AB457" s="102" t="s">
+      <c r="AA457" t="s">
+        <v>1201</v>
+      </c>
+      <c r="AB457" s="28" t="s">
         <v>1011</v>
       </c>
-      <c r="AC457" s="103" t="s">
+      <c r="AC457" s="20" t="s">
         <v>1038</v>
       </c>
-      <c r="AD457" s="101" t="s">
-        <v>785</v>
-      </c>
-      <c r="AE457" s="101" t="s">
+      <c r="AD457" s="33" t="s">
+        <v>786</v>
+      </c>
+      <c r="AE457" s="33" t="s">
         <v>1595</v>
       </c>
     </row>
-    <row r="458" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A458" s="70">
-        <v>40006</v>
-      </c>
-      <c r="B458" s="73" t="s">
-        <v>1581</v>
-      </c>
-      <c r="C458" s="73" t="s">
-        <v>1582</v>
-      </c>
-      <c r="D458" s="73" t="s">
+    <row r="458" spans="1:31" s="67" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A458" s="78">
+        <v>40008</v>
+      </c>
+      <c r="B458" s="67" t="s">
+        <v>1598</v>
+      </c>
+      <c r="C458" s="67" t="s">
+        <v>1602</v>
+      </c>
+      <c r="D458" s="63" t="s">
         <v>1278</v>
       </c>
-      <c r="E458" s="73" t="s">
+      <c r="E458" s="63" t="s">
         <v>1201</v>
       </c>
-      <c r="F458" s="73" t="s">
+      <c r="F458" s="63" t="s">
         <v>1201</v>
       </c>
-      <c r="G458" s="23">
-        <v>3</v>
-      </c>
-      <c r="H458" s="71" t="s">
-        <v>781</v>
-      </c>
-      <c r="I458" s="73" t="s">
-        <v>105</v>
-      </c>
-      <c r="J458">
-        <v>1</v>
-      </c>
-      <c r="K458">
-        <v>1</v>
-      </c>
-      <c r="M458">
+      <c r="G458" s="64">
+        <v>2</v>
+      </c>
+      <c r="H458" s="67" t="s">
+        <v>63</v>
+      </c>
+      <c r="I458" s="63" t="s">
+        <v>1606</v>
+      </c>
+      <c r="J458" s="67">
+        <v>1</v>
+      </c>
+      <c r="K458" s="67">
+        <v>1</v>
+      </c>
+      <c r="M458" s="67">
         <v>8</v>
       </c>
-      <c r="N458" t="s">
-        <v>1593</v>
-      </c>
-      <c r="O458" t="s">
-        <v>1594</v>
-      </c>
-      <c r="P458" s="38" t="s">
+      <c r="N458" s="67" t="s">
+        <v>1607</v>
+      </c>
+      <c r="O458" s="67" t="s">
+        <v>1612</v>
+      </c>
+      <c r="P458" s="67" t="s">
         <v>572</v>
       </c>
-      <c r="Q458" t="s">
-        <v>1587</v>
-      </c>
-      <c r="R458" s="33" t="s">
-        <v>95</v>
-      </c>
-      <c r="S458" s="71" t="s">
-        <v>784</v>
-      </c>
-      <c r="T458" s="31" t="s">
-        <v>967</v>
-      </c>
-      <c r="U458" t="s">
-        <v>1001</v>
-      </c>
-      <c r="V458" s="71" t="s">
-        <v>789</v>
-      </c>
-      <c r="W458" s="28" t="s">
-        <v>933</v>
-      </c>
-      <c r="X458" s="20" t="s">
-        <v>1038</v>
-      </c>
-      <c r="Y458" s="33" t="s">
-        <v>786</v>
-      </c>
-      <c r="Z458" s="33" t="s">
-        <v>1595</v>
-      </c>
-      <c r="AA458" s="71" t="s">
-        <v>787</v>
-      </c>
-      <c r="AB458" s="28" t="s">
-        <v>1011</v>
-      </c>
-      <c r="AC458" s="20" t="s">
-        <v>1038</v>
-      </c>
-      <c r="AD458" s="33" t="s">
-        <v>786</v>
-      </c>
-      <c r="AE458" s="33" t="s">
-        <v>1595</v>
+      <c r="Q458" s="67" t="s">
+        <v>1611</v>
+      </c>
+      <c r="R458" s="68" t="s">
+        <v>1613</v>
+      </c>
+      <c r="S458" s="67" t="s">
+        <v>1614</v>
+      </c>
+      <c r="T458" s="67" t="s">
+        <v>63</v>
+      </c>
+      <c r="U458" s="67" t="s">
+        <v>1615</v>
+      </c>
+      <c r="V458" s="67" t="s">
+        <v>1616</v>
+      </c>
+      <c r="W458" s="67" t="s">
+        <v>931</v>
+      </c>
+      <c r="X458" s="67" t="s">
+        <v>1617</v>
+      </c>
+      <c r="Y458" s="67" t="s">
+        <v>1618</v>
+      </c>
+      <c r="Z458" s="69" t="s">
+        <v>1048</v>
+      </c>
+      <c r="AA458" s="67" t="s">
+        <v>1616</v>
+      </c>
+      <c r="AB458" s="67" t="s">
+        <v>931</v>
+      </c>
+      <c r="AC458" s="67" t="s">
+        <v>1617</v>
+      </c>
+      <c r="AD458" s="67" t="s">
+        <v>1618</v>
+      </c>
+      <c r="AE458" s="69" t="s">
+        <v>1048</v>
       </c>
     </row>
     <row r="459" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A459" s="70">
-        <v>40007</v>
+        <v>40009</v>
       </c>
       <c r="B459" s="73" t="s">
-        <v>1583</v>
-      </c>
-      <c r="C459" s="73" t="s">
-        <v>1584</v>
+        <v>1599</v>
+      </c>
+      <c r="C459" s="67" t="s">
+        <v>1603</v>
       </c>
       <c r="D459" s="73" t="s">
         <v>1278</v>
@@ -52228,13 +52313,13 @@
         <v>1201</v>
       </c>
       <c r="G459" s="23">
-        <v>3</v>
-      </c>
-      <c r="H459" s="71" t="s">
-        <v>119</v>
+        <v>2</v>
+      </c>
+      <c r="H459" s="67" t="s">
+        <v>63</v>
       </c>
       <c r="I459" s="73" t="s">
-        <v>105</v>
+        <v>1606</v>
       </c>
       <c r="J459">
         <v>1</v>
@@ -52246,113 +52331,113 @@
         <v>8</v>
       </c>
       <c r="N459" t="s">
-        <v>1589</v>
+        <v>1608</v>
       </c>
       <c r="O459" t="s">
-        <v>1590</v>
+        <v>1612</v>
       </c>
       <c r="P459" s="38" t="s">
         <v>572</v>
       </c>
       <c r="Q459" t="s">
-        <v>1588</v>
-      </c>
-      <c r="R459" s="33" t="s">
-        <v>95</v>
-      </c>
-      <c r="S459" s="71" t="s">
-        <v>784</v>
-      </c>
-      <c r="T459" s="33" t="s">
-        <v>119</v>
-      </c>
-      <c r="U459" s="71" t="s">
-        <v>1585</v>
-      </c>
-      <c r="V459" s="71" t="s">
+        <v>1611</v>
+      </c>
+      <c r="R459" s="31" t="s">
+        <v>1613</v>
+      </c>
+      <c r="S459" t="s">
+        <v>1614</v>
+      </c>
+      <c r="T459" s="67" t="s">
+        <v>63</v>
+      </c>
+      <c r="U459" s="67" t="s">
+        <v>1615</v>
+      </c>
+      <c r="V459" t="s">
+        <v>1616</v>
+      </c>
+      <c r="W459" s="67" t="s">
+        <v>931</v>
+      </c>
+      <c r="X459" t="s">
+        <v>1617</v>
+      </c>
+      <c r="Y459" s="67" t="s">
+        <v>1618</v>
+      </c>
+      <c r="Z459" s="36" t="s">
+        <v>1048</v>
+      </c>
+      <c r="AA459" t="s">
+        <v>1616</v>
+      </c>
+      <c r="AB459" s="67" t="s">
+        <v>931</v>
+      </c>
+      <c r="AC459" t="s">
+        <v>1617</v>
+      </c>
+      <c r="AD459" s="67" t="s">
+        <v>1618</v>
+      </c>
+      <c r="AE459" s="36" t="s">
+        <v>1048</v>
+      </c>
+    </row>
+    <row r="460" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A460" s="70">
+        <v>40010</v>
+      </c>
+      <c r="B460" s="73" t="s">
+        <v>1600</v>
+      </c>
+      <c r="C460" s="67" t="s">
+        <v>1604</v>
+      </c>
+      <c r="D460" s="73" t="s">
+        <v>1278</v>
+      </c>
+      <c r="E460" s="73" t="s">
         <v>1201</v>
       </c>
-      <c r="W459" s="28" t="s">
-        <v>933</v>
-      </c>
-      <c r="X459" s="20" t="s">
-        <v>1038</v>
-      </c>
-      <c r="Y459" s="33" t="s">
-        <v>786</v>
-      </c>
-      <c r="Z459" s="33" t="s">
-        <v>1595</v>
-      </c>
-      <c r="AA459" t="s">
+      <c r="F460" s="73" t="s">
         <v>1201</v>
       </c>
-      <c r="AB459" s="28" t="s">
-        <v>1011</v>
-      </c>
-      <c r="AC459" s="20" t="s">
-        <v>1038</v>
-      </c>
-      <c r="AD459" s="33" t="s">
-        <v>786</v>
-      </c>
-      <c r="AE459" s="33" t="s">
-        <v>1595</v>
-      </c>
-    </row>
-    <row r="460" spans="1:31" s="67" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A460" s="78">
-        <v>40008</v>
-      </c>
-      <c r="B460" s="67" t="s">
-        <v>1598</v>
-      </c>
-      <c r="C460" s="67" t="s">
-        <v>1602</v>
-      </c>
-      <c r="D460" s="63" t="s">
-        <v>1278</v>
-      </c>
-      <c r="E460" s="63" t="s">
-        <v>1201</v>
-      </c>
-      <c r="F460" s="63" t="s">
-        <v>1201</v>
-      </c>
-      <c r="G460" s="64">
+      <c r="G460" s="23">
         <v>2</v>
       </c>
       <c r="H460" s="67" t="s">
         <v>63</v>
       </c>
-      <c r="I460" s="63" t="s">
+      <c r="I460" s="73" t="s">
         <v>1606</v>
       </c>
-      <c r="J460" s="67">
-        <v>1</v>
-      </c>
-      <c r="K460" s="67">
-        <v>1</v>
-      </c>
-      <c r="M460" s="67">
+      <c r="J460">
+        <v>1</v>
+      </c>
+      <c r="K460">
+        <v>1</v>
+      </c>
+      <c r="M460">
         <v>8</v>
       </c>
-      <c r="N460" s="67" t="s">
-        <v>1607</v>
+      <c r="N460" t="s">
+        <v>1609</v>
       </c>
       <c r="O460" s="67" t="s">
         <v>1612</v>
       </c>
-      <c r="P460" s="67" t="s">
+      <c r="P460" s="38" t="s">
         <v>572</v>
       </c>
-      <c r="Q460" s="67" t="s">
+      <c r="Q460" t="s">
         <v>1611</v>
       </c>
-      <c r="R460" s="68" t="s">
+      <c r="R460" s="31" t="s">
         <v>1613</v>
       </c>
-      <c r="S460" s="67" t="s">
+      <c r="S460" t="s">
         <v>1614</v>
       </c>
       <c r="T460" s="67" t="s">
@@ -52361,46 +52446,46 @@
       <c r="U460" s="67" t="s">
         <v>1615</v>
       </c>
-      <c r="V460" s="67" t="s">
+      <c r="V460" t="s">
         <v>1616</v>
       </c>
       <c r="W460" s="67" t="s">
         <v>931</v>
       </c>
-      <c r="X460" s="67" t="s">
+      <c r="X460" t="s">
         <v>1617</v>
       </c>
       <c r="Y460" s="67" t="s">
         <v>1618</v>
       </c>
-      <c r="Z460" s="69" t="s">
-        <v>1048</v>
-      </c>
-      <c r="AA460" s="67" t="s">
+      <c r="Z460" s="36" t="s">
+        <v>1048</v>
+      </c>
+      <c r="AA460" t="s">
         <v>1616</v>
       </c>
       <c r="AB460" s="67" t="s">
         <v>931</v>
       </c>
-      <c r="AC460" s="67" t="s">
+      <c r="AC460" t="s">
         <v>1617</v>
       </c>
       <c r="AD460" s="67" t="s">
         <v>1618</v>
       </c>
-      <c r="AE460" s="69" t="s">
+      <c r="AE460" s="36" t="s">
         <v>1048</v>
       </c>
     </row>
     <row r="461" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A461" s="70">
-        <v>40009</v>
+        <v>40011</v>
       </c>
       <c r="B461" s="73" t="s">
-        <v>1599</v>
+        <v>1601</v>
       </c>
       <c r="C461" s="67" t="s">
-        <v>1603</v>
+        <v>1605</v>
       </c>
       <c r="D461" s="73" t="s">
         <v>1278</v>
@@ -52430,7 +52515,7 @@
         <v>8</v>
       </c>
       <c r="N461" t="s">
-        <v>1608</v>
+        <v>1610</v>
       </c>
       <c r="O461" t="s">
         <v>1612</v>
@@ -52486,31 +52571,31 @@
     </row>
     <row r="462" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A462" s="70">
-        <v>40010</v>
-      </c>
-      <c r="B462" s="73" t="s">
-        <v>1600</v>
+        <v>40012</v>
+      </c>
+      <c r="B462" s="67" t="s">
+        <v>1623</v>
       </c>
       <c r="C462" s="67" t="s">
-        <v>1604</v>
-      </c>
-      <c r="D462" s="73" t="s">
+        <v>1602</v>
+      </c>
+      <c r="D462" s="63" t="s">
         <v>1278</v>
       </c>
-      <c r="E462" s="73" t="s">
+      <c r="E462" s="63" t="s">
         <v>1201</v>
       </c>
-      <c r="F462" s="73" t="s">
+      <c r="F462" s="63" t="s">
         <v>1201</v>
       </c>
-      <c r="G462" s="23">
+      <c r="G462" s="64">
         <v>2</v>
       </c>
       <c r="H462" s="67" t="s">
         <v>63</v>
       </c>
       <c r="I462" s="73" t="s">
-        <v>1606</v>
+        <v>106</v>
       </c>
       <c r="J462">
         <v>1</v>
@@ -52522,7 +52607,7 @@
         <v>8</v>
       </c>
       <c r="N462" t="s">
-        <v>1609</v>
+        <v>1627</v>
       </c>
       <c r="O462" s="67" t="s">
         <v>1612</v>
@@ -52534,9 +52619,9 @@
         <v>1611</v>
       </c>
       <c r="R462" s="31" t="s">
-        <v>1613</v>
-      </c>
-      <c r="S462" t="s">
+        <v>97</v>
+      </c>
+      <c r="S462" s="67" t="s">
         <v>1614</v>
       </c>
       <c r="T462" s="67" t="s">
@@ -52545,46 +52630,46 @@
       <c r="U462" s="67" t="s">
         <v>1615</v>
       </c>
-      <c r="V462" t="s">
+      <c r="V462" s="67" t="s">
         <v>1616</v>
       </c>
       <c r="W462" s="67" t="s">
         <v>931</v>
       </c>
-      <c r="X462" t="s">
+      <c r="X462" s="67" t="s">
         <v>1617</v>
       </c>
       <c r="Y462" s="67" t="s">
         <v>1618</v>
       </c>
-      <c r="Z462" s="36" t="s">
-        <v>1048</v>
-      </c>
-      <c r="AA462" t="s">
+      <c r="Z462" s="69" t="s">
+        <v>1048</v>
+      </c>
+      <c r="AA462" s="67" t="s">
         <v>1616</v>
       </c>
       <c r="AB462" s="67" t="s">
         <v>931</v>
       </c>
-      <c r="AC462" t="s">
+      <c r="AC462" s="67" t="s">
         <v>1617</v>
       </c>
       <c r="AD462" s="67" t="s">
         <v>1618</v>
       </c>
-      <c r="AE462" s="36" t="s">
+      <c r="AE462" s="69" t="s">
         <v>1048</v>
       </c>
     </row>
     <row r="463" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A463" s="70">
-        <v>40011</v>
-      </c>
-      <c r="B463" s="73" t="s">
-        <v>1601</v>
+        <v>40013</v>
+      </c>
+      <c r="B463" s="67" t="s">
+        <v>1624</v>
       </c>
       <c r="C463" s="67" t="s">
-        <v>1605</v>
+        <v>1603</v>
       </c>
       <c r="D463" s="73" t="s">
         <v>1278</v>
@@ -52602,7 +52687,7 @@
         <v>63</v>
       </c>
       <c r="I463" s="73" t="s">
-        <v>1606</v>
+        <v>106</v>
       </c>
       <c r="J463">
         <v>1</v>
@@ -52614,7 +52699,7 @@
         <v>8</v>
       </c>
       <c r="N463" t="s">
-        <v>1610</v>
+        <v>1628</v>
       </c>
       <c r="O463" t="s">
         <v>1612</v>
@@ -52626,7 +52711,7 @@
         <v>1611</v>
       </c>
       <c r="R463" s="31" t="s">
-        <v>1613</v>
+        <v>97</v>
       </c>
       <c r="S463" t="s">
         <v>1614</v>
@@ -52670,24 +52755,24 @@
     </row>
     <row r="464" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A464" s="70">
-        <v>40012</v>
+        <v>40014</v>
       </c>
       <c r="B464" s="67" t="s">
-        <v>1623</v>
+        <v>1625</v>
       </c>
       <c r="C464" s="67" t="s">
-        <v>1602</v>
-      </c>
-      <c r="D464" s="63" t="s">
+        <v>1604</v>
+      </c>
+      <c r="D464" s="73" t="s">
         <v>1278</v>
       </c>
-      <c r="E464" s="63" t="s">
+      <c r="E464" s="73" t="s">
         <v>1201</v>
       </c>
-      <c r="F464" s="63" t="s">
+      <c r="F464" s="73" t="s">
         <v>1201</v>
       </c>
-      <c r="G464" s="64">
+      <c r="G464" s="23">
         <v>2</v>
       </c>
       <c r="H464" s="67" t="s">
@@ -52706,7 +52791,7 @@
         <v>8</v>
       </c>
       <c r="N464" t="s">
-        <v>1627</v>
+        <v>1629</v>
       </c>
       <c r="O464" s="67" t="s">
         <v>1612</v>
@@ -52720,7 +52805,7 @@
       <c r="R464" s="31" t="s">
         <v>97</v>
       </c>
-      <c r="S464" s="67" t="s">
+      <c r="S464" t="s">
         <v>1614</v>
       </c>
       <c r="T464" s="67" t="s">
@@ -52729,46 +52814,46 @@
       <c r="U464" s="67" t="s">
         <v>1615</v>
       </c>
-      <c r="V464" s="67" t="s">
+      <c r="V464" t="s">
         <v>1616</v>
       </c>
       <c r="W464" s="67" t="s">
         <v>931</v>
       </c>
-      <c r="X464" s="67" t="s">
+      <c r="X464" t="s">
         <v>1617</v>
       </c>
       <c r="Y464" s="67" t="s">
         <v>1618</v>
       </c>
-      <c r="Z464" s="69" t="s">
-        <v>1048</v>
-      </c>
-      <c r="AA464" s="67" t="s">
+      <c r="Z464" s="36" t="s">
+        <v>1048</v>
+      </c>
+      <c r="AA464" t="s">
         <v>1616</v>
       </c>
       <c r="AB464" s="67" t="s">
         <v>931</v>
       </c>
-      <c r="AC464" s="67" t="s">
+      <c r="AC464" t="s">
         <v>1617</v>
       </c>
       <c r="AD464" s="67" t="s">
         <v>1618</v>
       </c>
-      <c r="AE464" s="69" t="s">
+      <c r="AE464" s="36" t="s">
         <v>1048</v>
       </c>
     </row>
     <row r="465" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A465" s="70">
-        <v>40013</v>
+        <v>40015</v>
       </c>
       <c r="B465" s="67" t="s">
-        <v>1624</v>
+        <v>1626</v>
       </c>
       <c r="C465" s="67" t="s">
-        <v>1603</v>
+        <v>1605</v>
       </c>
       <c r="D465" s="73" t="s">
         <v>1278</v>
@@ -52798,7 +52883,7 @@
         <v>8</v>
       </c>
       <c r="N465" t="s">
-        <v>1628</v>
+        <v>1630</v>
       </c>
       <c r="O465" t="s">
         <v>1612</v>
@@ -52852,26 +52937,26 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="466" spans="1:31" x14ac:dyDescent="0.2">
+    <row r="466" spans="1:31" s="67" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A466" s="70">
-        <v>40014</v>
+        <v>40016</v>
       </c>
       <c r="B466" s="67" t="s">
-        <v>1625</v>
+        <v>1619</v>
       </c>
       <c r="C466" s="67" t="s">
-        <v>1604</v>
-      </c>
-      <c r="D466" s="73" t="s">
+        <v>1602</v>
+      </c>
+      <c r="D466" s="63" t="s">
         <v>1278</v>
       </c>
-      <c r="E466" s="73" t="s">
+      <c r="E466" s="63" t="s">
         <v>1201</v>
       </c>
-      <c r="F466" s="73" t="s">
+      <c r="F466" s="63" t="s">
         <v>1201</v>
       </c>
-      <c r="G466" s="23">
+      <c r="G466" s="64">
         <v>2</v>
       </c>
       <c r="H466" s="67" t="s">
@@ -52880,31 +52965,31 @@
       <c r="I466" s="73" t="s">
         <v>106</v>
       </c>
-      <c r="J466">
-        <v>1</v>
-      </c>
-      <c r="K466">
-        <v>1</v>
-      </c>
-      <c r="M466">
+      <c r="J466" s="67">
+        <v>1</v>
+      </c>
+      <c r="K466" s="67">
+        <v>1</v>
+      </c>
+      <c r="M466" s="67">
         <v>8</v>
       </c>
-      <c r="N466" t="s">
-        <v>1629</v>
+      <c r="N466" s="67" t="s">
+        <v>1607</v>
       </c>
       <c r="O466" s="67" t="s">
         <v>1612</v>
       </c>
-      <c r="P466" s="38" t="s">
+      <c r="P466" s="67" t="s">
         <v>572</v>
       </c>
-      <c r="Q466" t="s">
+      <c r="Q466" s="67" t="s">
         <v>1611</v>
       </c>
       <c r="R466" s="31" t="s">
         <v>97</v>
       </c>
-      <c r="S466" t="s">
+      <c r="S466" s="67" t="s">
         <v>1614</v>
       </c>
       <c r="T466" s="67" t="s">
@@ -52913,46 +52998,46 @@
       <c r="U466" s="67" t="s">
         <v>1615</v>
       </c>
-      <c r="V466" t="s">
+      <c r="V466" s="67" t="s">
         <v>1616</v>
       </c>
       <c r="W466" s="67" t="s">
         <v>931</v>
       </c>
-      <c r="X466" t="s">
+      <c r="X466" s="67" t="s">
         <v>1617</v>
       </c>
       <c r="Y466" s="67" t="s">
         <v>1618</v>
       </c>
-      <c r="Z466" s="36" t="s">
-        <v>1048</v>
-      </c>
-      <c r="AA466" t="s">
+      <c r="Z466" s="69" t="s">
+        <v>1048</v>
+      </c>
+      <c r="AA466" s="67" t="s">
         <v>1616</v>
       </c>
       <c r="AB466" s="67" t="s">
         <v>931</v>
       </c>
-      <c r="AC466" t="s">
+      <c r="AC466" s="67" t="s">
         <v>1617</v>
       </c>
       <c r="AD466" s="67" t="s">
         <v>1618</v>
       </c>
-      <c r="AE466" s="36" t="s">
+      <c r="AE466" s="69" t="s">
         <v>1048</v>
       </c>
     </row>
     <row r="467" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A467" s="70">
-        <v>40015</v>
-      </c>
-      <c r="B467" s="67" t="s">
-        <v>1626</v>
+        <v>40017</v>
+      </c>
+      <c r="B467" s="73" t="s">
+        <v>1620</v>
       </c>
       <c r="C467" s="67" t="s">
-        <v>1605</v>
+        <v>1603</v>
       </c>
       <c r="D467" s="73" t="s">
         <v>1278</v>
@@ -52982,7 +53067,7 @@
         <v>8</v>
       </c>
       <c r="N467" t="s">
-        <v>1630</v>
+        <v>1608</v>
       </c>
       <c r="O467" t="s">
         <v>1612</v>
@@ -53036,26 +53121,26 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="468" spans="1:31" s="67" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="468" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A468" s="70">
-        <v>40016</v>
-      </c>
-      <c r="B468" s="67" t="s">
-        <v>1619</v>
+        <v>40018</v>
+      </c>
+      <c r="B468" s="73" t="s">
+        <v>1621</v>
       </c>
       <c r="C468" s="67" t="s">
-        <v>1602</v>
-      </c>
-      <c r="D468" s="63" t="s">
+        <v>1604</v>
+      </c>
+      <c r="D468" s="73" t="s">
         <v>1278</v>
       </c>
-      <c r="E468" s="63" t="s">
+      <c r="E468" s="73" t="s">
         <v>1201</v>
       </c>
-      <c r="F468" s="63" t="s">
+      <c r="F468" s="73" t="s">
         <v>1201</v>
       </c>
-      <c r="G468" s="64">
+      <c r="G468" s="23">
         <v>2</v>
       </c>
       <c r="H468" s="67" t="s">
@@ -53064,31 +53149,31 @@
       <c r="I468" s="73" t="s">
         <v>106</v>
       </c>
-      <c r="J468" s="67">
-        <v>1</v>
-      </c>
-      <c r="K468" s="67">
-        <v>1</v>
-      </c>
-      <c r="M468" s="67">
+      <c r="J468">
+        <v>1</v>
+      </c>
+      <c r="K468">
+        <v>1</v>
+      </c>
+      <c r="M468">
         <v>8</v>
       </c>
-      <c r="N468" s="67" t="s">
-        <v>1607</v>
+      <c r="N468" t="s">
+        <v>1609</v>
       </c>
       <c r="O468" s="67" t="s">
         <v>1612</v>
       </c>
-      <c r="P468" s="67" t="s">
+      <c r="P468" s="38" t="s">
         <v>572</v>
       </c>
-      <c r="Q468" s="67" t="s">
+      <c r="Q468" t="s">
         <v>1611</v>
       </c>
       <c r="R468" s="31" t="s">
         <v>97</v>
       </c>
-      <c r="S468" s="67" t="s">
+      <c r="S468" t="s">
         <v>1614</v>
       </c>
       <c r="T468" s="67" t="s">
@@ -53097,46 +53182,46 @@
       <c r="U468" s="67" t="s">
         <v>1615</v>
       </c>
-      <c r="V468" s="67" t="s">
+      <c r="V468" t="s">
         <v>1616</v>
       </c>
       <c r="W468" s="67" t="s">
         <v>931</v>
       </c>
-      <c r="X468" s="67" t="s">
+      <c r="X468" t="s">
         <v>1617</v>
       </c>
       <c r="Y468" s="67" t="s">
         <v>1618</v>
       </c>
-      <c r="Z468" s="69" t="s">
-        <v>1048</v>
-      </c>
-      <c r="AA468" s="67" t="s">
+      <c r="Z468" s="36" t="s">
+        <v>1048</v>
+      </c>
+      <c r="AA468" t="s">
         <v>1616</v>
       </c>
       <c r="AB468" s="67" t="s">
         <v>931</v>
       </c>
-      <c r="AC468" s="67" t="s">
+      <c r="AC468" t="s">
         <v>1617</v>
       </c>
       <c r="AD468" s="67" t="s">
         <v>1618</v>
       </c>
-      <c r="AE468" s="69" t="s">
+      <c r="AE468" s="36" t="s">
         <v>1048</v>
       </c>
     </row>
     <row r="469" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A469" s="70">
-        <v>40017</v>
+        <v>40019</v>
       </c>
       <c r="B469" s="73" t="s">
-        <v>1620</v>
+        <v>1622</v>
       </c>
       <c r="C469" s="67" t="s">
-        <v>1603</v>
+        <v>1605</v>
       </c>
       <c r="D469" s="73" t="s">
         <v>1278</v>
@@ -53166,7 +53251,7 @@
         <v>8</v>
       </c>
       <c r="N469" t="s">
-        <v>1608</v>
+        <v>1610</v>
       </c>
       <c r="O469" t="s">
         <v>1612</v>
@@ -53222,13 +53307,13 @@
     </row>
     <row r="470" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A470" s="70">
-        <v>40018</v>
+        <v>40020</v>
       </c>
       <c r="B470" s="73" t="s">
-        <v>1621</v>
-      </c>
-      <c r="C470" s="67" t="s">
-        <v>1604</v>
+        <v>1631</v>
+      </c>
+      <c r="C470" t="s">
+        <v>1640</v>
       </c>
       <c r="D470" s="73" t="s">
         <v>1278</v>
@@ -53242,14 +53327,14 @@
       <c r="G470" s="23">
         <v>2</v>
       </c>
-      <c r="H470" s="67" t="s">
-        <v>63</v>
+      <c r="H470" s="71" t="s">
+        <v>110</v>
       </c>
       <c r="I470" s="73" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="J470">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K470">
         <v>1</v>
@@ -53258,55 +53343,55 @@
         <v>8</v>
       </c>
       <c r="N470" t="s">
-        <v>1609</v>
-      </c>
-      <c r="O470" s="67" t="s">
-        <v>1612</v>
+        <v>468</v>
+      </c>
+      <c r="O470" t="s">
+        <v>477</v>
       </c>
       <c r="P470" s="38" t="s">
         <v>572</v>
       </c>
       <c r="Q470" t="s">
-        <v>1611</v>
-      </c>
-      <c r="R470" s="31" t="s">
-        <v>97</v>
+        <v>479</v>
+      </c>
+      <c r="R470" s="107" t="s">
+        <v>892</v>
       </c>
       <c r="S470" t="s">
-        <v>1614</v>
-      </c>
-      <c r="T470" s="67" t="s">
-        <v>63</v>
-      </c>
-      <c r="U470" s="67" t="s">
-        <v>1615</v>
-      </c>
-      <c r="V470" t="s">
-        <v>1616</v>
-      </c>
-      <c r="W470" s="67" t="s">
-        <v>931</v>
-      </c>
-      <c r="X470" t="s">
-        <v>1617</v>
-      </c>
-      <c r="Y470" s="67" t="s">
-        <v>1618</v>
+        <v>12</v>
+      </c>
+      <c r="T470" s="51" t="s">
+        <v>963</v>
+      </c>
+      <c r="U470" s="23" t="s">
+        <v>1003</v>
+      </c>
+      <c r="V470" s="108" t="s">
+        <v>13</v>
+      </c>
+      <c r="W470" s="109" t="s">
+        <v>927</v>
+      </c>
+      <c r="X470" s="59" t="s">
+        <v>1017</v>
+      </c>
+      <c r="Y470" s="36" t="s">
+        <v>1650</v>
       </c>
       <c r="Z470" s="36" t="s">
         <v>1048</v>
       </c>
-      <c r="AA470" t="s">
-        <v>1616</v>
-      </c>
-      <c r="AB470" s="67" t="s">
-        <v>931</v>
-      </c>
-      <c r="AC470" t="s">
-        <v>1617</v>
-      </c>
-      <c r="AD470" s="67" t="s">
-        <v>1618</v>
+      <c r="AA470" s="110" t="s">
+        <v>113</v>
+      </c>
+      <c r="AB470" s="111" t="s">
+        <v>937</v>
+      </c>
+      <c r="AC470" s="60" t="s">
+        <v>1017</v>
+      </c>
+      <c r="AD470" s="36" t="s">
+        <v>1649</v>
       </c>
       <c r="AE470" s="36" t="s">
         <v>1048</v>
@@ -53314,13 +53399,13 @@
     </row>
     <row r="471" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A471" s="70">
-        <v>40019</v>
+        <v>40021</v>
       </c>
       <c r="B471" s="73" t="s">
-        <v>1622</v>
-      </c>
-      <c r="C471" s="67" t="s">
-        <v>1605</v>
+        <v>1632</v>
+      </c>
+      <c r="C471" t="s">
+        <v>1641</v>
       </c>
       <c r="D471" s="73" t="s">
         <v>1278</v>
@@ -53334,14 +53419,14 @@
       <c r="G471" s="23">
         <v>2</v>
       </c>
-      <c r="H471" s="67" t="s">
-        <v>63</v>
+      <c r="H471" s="71" t="s">
+        <v>110</v>
       </c>
       <c r="I471" s="73" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="J471">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K471">
         <v>1</v>
@@ -53350,55 +53435,55 @@
         <v>8</v>
       </c>
       <c r="N471" t="s">
-        <v>1610</v>
+        <v>469</v>
       </c>
       <c r="O471" t="s">
-        <v>1612</v>
+        <v>477</v>
       </c>
       <c r="P471" s="38" t="s">
         <v>572</v>
       </c>
       <c r="Q471" t="s">
-        <v>1611</v>
-      </c>
-      <c r="R471" s="31" t="s">
-        <v>97</v>
+        <v>479</v>
+      </c>
+      <c r="R471" s="82" t="s">
+        <v>892</v>
       </c>
       <c r="S471" t="s">
-        <v>1614</v>
-      </c>
-      <c r="T471" s="67" t="s">
-        <v>63</v>
-      </c>
-      <c r="U471" s="67" t="s">
-        <v>1615</v>
-      </c>
-      <c r="V471" t="s">
-        <v>1616</v>
-      </c>
-      <c r="W471" s="67" t="s">
-        <v>931</v>
-      </c>
-      <c r="X471" t="s">
-        <v>1617</v>
-      </c>
-      <c r="Y471" s="67" t="s">
-        <v>1618</v>
+        <v>12</v>
+      </c>
+      <c r="T471" s="51" t="s">
+        <v>963</v>
+      </c>
+      <c r="U471" s="23" t="s">
+        <v>1003</v>
+      </c>
+      <c r="V471" s="108" t="s">
+        <v>13</v>
+      </c>
+      <c r="W471" s="109" t="s">
+        <v>927</v>
+      </c>
+      <c r="X471" s="59" t="s">
+        <v>1017</v>
+      </c>
+      <c r="Y471" s="36" t="s">
+        <v>1650</v>
       </c>
       <c r="Z471" s="36" t="s">
         <v>1048</v>
       </c>
-      <c r="AA471" t="s">
-        <v>1616</v>
-      </c>
-      <c r="AB471" s="67" t="s">
-        <v>931</v>
-      </c>
-      <c r="AC471" t="s">
-        <v>1617</v>
-      </c>
-      <c r="AD471" s="67" t="s">
-        <v>1618</v>
+      <c r="AA471" s="110" t="s">
+        <v>113</v>
+      </c>
+      <c r="AB471" s="111" t="s">
+        <v>937</v>
+      </c>
+      <c r="AC471" s="60" t="s">
+        <v>1017</v>
+      </c>
+      <c r="AD471" s="36" t="s">
+        <v>1649</v>
       </c>
       <c r="AE471" s="36" t="s">
         <v>1048</v>
@@ -53406,13 +53491,13 @@
     </row>
     <row r="472" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A472" s="70">
-        <v>40020</v>
+        <v>40022</v>
       </c>
       <c r="B472" s="73" t="s">
-        <v>1631</v>
+        <v>1633</v>
       </c>
       <c r="C472" t="s">
-        <v>1640</v>
+        <v>1642</v>
       </c>
       <c r="D472" s="73" t="s">
         <v>1278</v>
@@ -53442,7 +53527,7 @@
         <v>8</v>
       </c>
       <c r="N472" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="O472" t="s">
         <v>477</v>
@@ -53453,7 +53538,7 @@
       <c r="Q472" t="s">
         <v>479</v>
       </c>
-      <c r="R472" s="107" t="s">
+      <c r="R472" s="82" t="s">
         <v>892</v>
       </c>
       <c r="S472" t="s">
@@ -53498,13 +53583,13 @@
     </row>
     <row r="473" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A473" s="70">
-        <v>40021</v>
+        <v>40023</v>
       </c>
       <c r="B473" s="73" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="C473" t="s">
-        <v>1641</v>
+        <v>1643</v>
       </c>
       <c r="D473" s="73" t="s">
         <v>1278</v>
@@ -53534,7 +53619,7 @@
         <v>8</v>
       </c>
       <c r="N473" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="O473" t="s">
         <v>477</v>
@@ -53590,13 +53675,13 @@
     </row>
     <row r="474" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A474" s="70">
-        <v>40022</v>
+        <v>40024</v>
       </c>
       <c r="B474" s="73" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="C474" t="s">
-        <v>1642</v>
+        <v>1644</v>
       </c>
       <c r="D474" s="73" t="s">
         <v>1278</v>
@@ -53626,7 +53711,7 @@
         <v>8</v>
       </c>
       <c r="N474" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="O474" t="s">
         <v>477</v>
@@ -53682,13 +53767,13 @@
     </row>
     <row r="475" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A475" s="70">
-        <v>40023</v>
+        <v>40025</v>
       </c>
       <c r="B475" s="73" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="C475" t="s">
-        <v>1643</v>
+        <v>1645</v>
       </c>
       <c r="D475" s="73" t="s">
         <v>1278</v>
@@ -53718,7 +53803,7 @@
         <v>8</v>
       </c>
       <c r="N475" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="O475" t="s">
         <v>477</v>
@@ -53774,13 +53859,13 @@
     </row>
     <row r="476" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A476" s="70">
-        <v>40024</v>
+        <v>40026</v>
       </c>
       <c r="B476" s="73" t="s">
-        <v>1635</v>
+        <v>1637</v>
       </c>
       <c r="C476" t="s">
-        <v>1644</v>
+        <v>1646</v>
       </c>
       <c r="D476" s="73" t="s">
         <v>1278</v>
@@ -53810,7 +53895,7 @@
         <v>8</v>
       </c>
       <c r="N476" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="O476" t="s">
         <v>477</v>
@@ -53866,13 +53951,13 @@
     </row>
     <row r="477" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A477" s="70">
-        <v>40025</v>
+        <v>40027</v>
       </c>
       <c r="B477" s="73" t="s">
-        <v>1636</v>
+        <v>1638</v>
       </c>
       <c r="C477" t="s">
-        <v>1645</v>
+        <v>1647</v>
       </c>
       <c r="D477" s="73" t="s">
         <v>1278</v>
@@ -53902,7 +53987,7 @@
         <v>8</v>
       </c>
       <c r="N477" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="O477" t="s">
         <v>477</v>
@@ -53958,13 +54043,13 @@
     </row>
     <row r="478" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A478" s="70">
-        <v>40026</v>
+        <v>40028</v>
       </c>
       <c r="B478" s="73" t="s">
-        <v>1637</v>
+        <v>1639</v>
       </c>
       <c r="C478" t="s">
-        <v>1646</v>
+        <v>1648</v>
       </c>
       <c r="D478" s="73" t="s">
         <v>1278</v>
@@ -53994,7 +54079,7 @@
         <v>8</v>
       </c>
       <c r="N478" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="O478" t="s">
         <v>477</v>
@@ -54050,16 +54135,16 @@
     </row>
     <row r="479" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A479" s="70">
-        <v>40027</v>
+        <v>40029</v>
       </c>
       <c r="B479" s="73" t="s">
-        <v>1638</v>
+        <v>1651</v>
       </c>
       <c r="C479" t="s">
-        <v>1647</v>
+        <v>1361</v>
       </c>
       <c r="D479" s="73" t="s">
-        <v>1278</v>
+        <v>1277</v>
       </c>
       <c r="E479" s="73" t="s">
         <v>1201</v>
@@ -54068,16 +54153,16 @@
         <v>1201</v>
       </c>
       <c r="G479" s="23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H479" s="71" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="I479" s="73" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
       <c r="J479">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K479">
         <v>1</v>
@@ -54086,164 +54171,164 @@
         <v>8</v>
       </c>
       <c r="N479" t="s">
-        <v>475</v>
+        <v>1654</v>
       </c>
       <c r="O479" t="s">
-        <v>477</v>
-      </c>
-      <c r="P479" s="38" t="s">
         <v>572</v>
       </c>
+      <c r="P479" s="70" t="s">
+        <v>572</v>
+      </c>
       <c r="Q479" t="s">
-        <v>479</v>
-      </c>
-      <c r="R479" s="82" t="s">
-        <v>892</v>
+        <v>1655</v>
+      </c>
+      <c r="R479" s="107" t="s">
+        <v>128</v>
       </c>
       <c r="S479" t="s">
-        <v>12</v>
-      </c>
-      <c r="T479" s="51" t="s">
-        <v>963</v>
+        <v>129</v>
+      </c>
+      <c r="T479" s="31" t="s">
+        <v>126</v>
       </c>
       <c r="U479" s="23" t="s">
-        <v>1003</v>
+        <v>979</v>
       </c>
       <c r="V479" s="108" t="s">
-        <v>13</v>
+        <v>1652</v>
       </c>
       <c r="W479" s="109" t="s">
-        <v>927</v>
+        <v>929</v>
       </c>
       <c r="X479" s="59" t="s">
-        <v>1017</v>
+        <v>1024</v>
       </c>
       <c r="Y479" s="36" t="s">
-        <v>1650</v>
-      </c>
-      <c r="Z479" s="36" t="s">
-        <v>1048</v>
+        <v>131</v>
+      </c>
+      <c r="Z479" s="110" t="s">
+        <v>1653</v>
       </c>
       <c r="AA479" s="110" t="s">
-        <v>113</v>
+        <v>1652</v>
       </c>
       <c r="AB479" s="111" t="s">
-        <v>937</v>
+        <v>929</v>
       </c>
       <c r="AC479" s="60" t="s">
-        <v>1017</v>
+        <v>1042</v>
       </c>
       <c r="AD479" s="36" t="s">
-        <v>1649</v>
+        <v>132</v>
       </c>
       <c r="AE479" s="36" t="s">
-        <v>1048</v>
+        <v>1653</v>
       </c>
     </row>
-    <row r="480" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A480" s="70">
-        <v>40028</v>
-      </c>
-      <c r="B480" s="73" t="s">
-        <v>1639</v>
-      </c>
-      <c r="C480" t="s">
-        <v>1648</v>
-      </c>
-      <c r="D480" s="73" t="s">
+    <row r="480" spans="1:31" s="67" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A480" s="78">
+        <v>40030</v>
+      </c>
+      <c r="B480" s="63" t="s">
+        <v>1668</v>
+      </c>
+      <c r="C480" s="67" t="s">
+        <v>1670</v>
+      </c>
+      <c r="D480" s="63" t="s">
         <v>1278</v>
       </c>
-      <c r="E480" s="73" t="s">
+      <c r="E480" s="63" t="s">
         <v>1201</v>
       </c>
-      <c r="F480" s="73" t="s">
+      <c r="F480" s="63" t="s">
         <v>1201</v>
       </c>
-      <c r="G480" s="23">
-        <v>2</v>
-      </c>
-      <c r="H480" s="71" t="s">
-        <v>110</v>
-      </c>
-      <c r="I480" s="73" t="s">
+      <c r="G480" s="64">
+        <v>2</v>
+      </c>
+      <c r="H480" s="63" t="s">
+        <v>1656</v>
+      </c>
+      <c r="I480" s="63" t="s">
         <v>104</v>
       </c>
-      <c r="J480">
-        <v>3</v>
-      </c>
-      <c r="K480">
-        <v>1</v>
-      </c>
-      <c r="M480">
+      <c r="J480" s="67">
+        <v>1</v>
+      </c>
+      <c r="K480" s="67">
+        <v>1</v>
+      </c>
+      <c r="M480" s="67">
         <v>8</v>
       </c>
-      <c r="N480" t="s">
-        <v>476</v>
-      </c>
-      <c r="O480" t="s">
-        <v>477</v>
-      </c>
-      <c r="P480" s="38" t="s">
+      <c r="N480" s="67" t="s">
+        <v>1666</v>
+      </c>
+      <c r="O480" s="67" t="s">
+        <v>1667</v>
+      </c>
+      <c r="P480" s="78" t="s">
         <v>572</v>
       </c>
-      <c r="Q480" t="s">
-        <v>479</v>
-      </c>
-      <c r="R480" s="82" t="s">
-        <v>892</v>
-      </c>
-      <c r="S480" t="s">
-        <v>12</v>
-      </c>
-      <c r="T480" s="51" t="s">
-        <v>963</v>
-      </c>
-      <c r="U480" s="23" t="s">
-        <v>1003</v>
-      </c>
-      <c r="V480" s="108" t="s">
-        <v>13</v>
-      </c>
-      <c r="W480" s="109" t="s">
-        <v>927</v>
-      </c>
-      <c r="X480" s="59" t="s">
-        <v>1017</v>
-      </c>
-      <c r="Y480" s="36" t="s">
-        <v>1650</v>
-      </c>
-      <c r="Z480" s="36" t="s">
-        <v>1048</v>
-      </c>
-      <c r="AA480" s="110" t="s">
-        <v>113</v>
-      </c>
-      <c r="AB480" s="111" t="s">
-        <v>937</v>
-      </c>
-      <c r="AC480" s="60" t="s">
-        <v>1017</v>
-      </c>
-      <c r="AD480" s="36" t="s">
-        <v>1649</v>
-      </c>
-      <c r="AE480" s="36" t="s">
+      <c r="Q480" s="67" t="s">
+        <v>1674</v>
+      </c>
+      <c r="R480" s="112" t="s">
+        <v>1658</v>
+      </c>
+      <c r="S480" s="67" t="s">
+        <v>1659</v>
+      </c>
+      <c r="T480" s="83" t="s">
+        <v>1656</v>
+      </c>
+      <c r="U480" s="64" t="s">
+        <v>1001</v>
+      </c>
+      <c r="V480" s="113" t="s">
+        <v>1201</v>
+      </c>
+      <c r="W480" s="102" t="s">
+        <v>933</v>
+      </c>
+      <c r="X480" s="67" t="s">
+        <v>1660</v>
+      </c>
+      <c r="Y480" s="69" t="s">
+        <v>1661</v>
+      </c>
+      <c r="Z480" s="69" t="s">
+        <v>1048</v>
+      </c>
+      <c r="AA480" s="114" t="s">
+        <v>1201</v>
+      </c>
+      <c r="AB480" s="102" t="s">
+        <v>1011</v>
+      </c>
+      <c r="AC480" s="67" t="s">
+        <v>1662</v>
+      </c>
+      <c r="AD480" s="69" t="s">
+        <v>1663</v>
+      </c>
+      <c r="AE480" s="69" t="s">
         <v>1048</v>
       </c>
     </row>
     <row r="481" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A481" s="70">
-        <v>40029</v>
+        <v>40031</v>
       </c>
       <c r="B481" s="73" t="s">
-        <v>1651</v>
+        <v>1669</v>
       </c>
       <c r="C481" t="s">
-        <v>1361</v>
+        <v>1671</v>
       </c>
       <c r="D481" s="73" t="s">
-        <v>1277</v>
+        <v>1278</v>
       </c>
       <c r="E481" s="73" t="s">
         <v>1201</v>
@@ -54252,13 +54337,13 @@
         <v>1201</v>
       </c>
       <c r="G481" s="23">
-        <v>3</v>
-      </c>
-      <c r="H481" s="71" t="s">
-        <v>126</v>
+        <v>2</v>
+      </c>
+      <c r="H481" s="73" t="s">
+        <v>1657</v>
       </c>
       <c r="I481" s="73" t="s">
-        <v>127</v>
+        <v>104</v>
       </c>
       <c r="J481">
         <v>1</v>
@@ -54270,158 +54355,158 @@
         <v>8</v>
       </c>
       <c r="N481" t="s">
-        <v>1654</v>
+        <v>1672</v>
       </c>
       <c r="O481" t="s">
-        <v>572</v>
+        <v>1673</v>
       </c>
       <c r="P481" s="70" t="s">
         <v>572</v>
       </c>
       <c r="Q481" t="s">
-        <v>1655</v>
+        <v>1665</v>
       </c>
       <c r="R481" s="107" t="s">
-        <v>128</v>
+        <v>1658</v>
       </c>
       <c r="S481" t="s">
-        <v>129</v>
-      </c>
-      <c r="T481" s="31" t="s">
-        <v>126</v>
+        <v>1659</v>
+      </c>
+      <c r="T481" s="51" t="s">
+        <v>1657</v>
       </c>
       <c r="U481" s="23" t="s">
-        <v>979</v>
+        <v>1664</v>
       </c>
       <c r="V481" s="108" t="s">
-        <v>1652</v>
-      </c>
-      <c r="W481" s="109" t="s">
-        <v>929</v>
-      </c>
-      <c r="X481" s="59" t="s">
-        <v>1024</v>
+        <v>1201</v>
+      </c>
+      <c r="W481" s="102" t="s">
+        <v>933</v>
+      </c>
+      <c r="X481" t="s">
+        <v>1660</v>
       </c>
       <c r="Y481" s="36" t="s">
-        <v>131</v>
-      </c>
-      <c r="Z481" s="110" t="s">
-        <v>1653</v>
+        <v>1661</v>
+      </c>
+      <c r="Z481" s="36" t="s">
+        <v>1048</v>
       </c>
       <c r="AA481" s="110" t="s">
-        <v>1652</v>
-      </c>
-      <c r="AB481" s="111" t="s">
-        <v>929</v>
-      </c>
-      <c r="AC481" s="60" t="s">
-        <v>1042</v>
+        <v>1201</v>
+      </c>
+      <c r="AB481" s="102" t="s">
+        <v>1011</v>
+      </c>
+      <c r="AC481" t="s">
+        <v>1662</v>
       </c>
       <c r="AD481" s="36" t="s">
-        <v>132</v>
+        <v>1663</v>
       </c>
       <c r="AE481" s="36" t="s">
-        <v>1653</v>
+        <v>1048</v>
       </c>
     </row>
-    <row r="482" spans="1:31" s="67" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A482" s="78">
-        <v>40030</v>
-      </c>
-      <c r="B482" s="63" t="s">
-        <v>1668</v>
-      </c>
-      <c r="C482" s="67" t="s">
+    <row r="482" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A482" s="70">
+        <v>40032</v>
+      </c>
+      <c r="B482" s="73" t="s">
+        <v>1677</v>
+      </c>
+      <c r="C482" t="s">
         <v>1670</v>
       </c>
-      <c r="D482" s="63" t="s">
+      <c r="D482" s="73" t="s">
         <v>1278</v>
       </c>
-      <c r="E482" s="63" t="s">
+      <c r="E482" s="73" t="s">
         <v>1201</v>
       </c>
-      <c r="F482" s="63" t="s">
+      <c r="F482" s="73" t="s">
         <v>1201</v>
       </c>
-      <c r="G482" s="64">
-        <v>2</v>
-      </c>
-      <c r="H482" s="63" t="s">
-        <v>1656</v>
-      </c>
-      <c r="I482" s="63" t="s">
+      <c r="G482" s="23">
+        <v>2</v>
+      </c>
+      <c r="H482" s="73" t="s">
+        <v>1675</v>
+      </c>
+      <c r="I482" s="73" t="s">
         <v>104</v>
       </c>
-      <c r="J482" s="67">
-        <v>1</v>
-      </c>
-      <c r="K482" s="67">
-        <v>1</v>
-      </c>
-      <c r="M482" s="67">
+      <c r="J482">
+        <v>1</v>
+      </c>
+      <c r="K482">
+        <v>1</v>
+      </c>
+      <c r="M482">
         <v>8</v>
       </c>
-      <c r="N482" s="67" t="s">
+      <c r="N482" t="s">
         <v>1666</v>
       </c>
-      <c r="O482" s="67" t="s">
+      <c r="O482" t="s">
         <v>1667</v>
       </c>
-      <c r="P482" s="78" t="s">
+      <c r="P482" s="70" t="s">
         <v>572</v>
       </c>
-      <c r="Q482" s="67" t="s">
+      <c r="Q482" t="s">
         <v>1674</v>
       </c>
-      <c r="R482" s="112" t="s">
+      <c r="R482" s="107" t="s">
         <v>1658</v>
       </c>
-      <c r="S482" s="67" t="s">
+      <c r="S482" t="s">
         <v>1659</v>
       </c>
-      <c r="T482" s="83" t="s">
-        <v>1656</v>
-      </c>
-      <c r="U482" s="64" t="s">
+      <c r="T482" s="51" t="s">
+        <v>146</v>
+      </c>
+      <c r="U482" s="23" t="s">
         <v>1001</v>
       </c>
-      <c r="V482" s="113" t="s">
+      <c r="V482" s="108" t="s">
         <v>1201</v>
       </c>
       <c r="W482" s="102" t="s">
         <v>933</v>
       </c>
-      <c r="X482" s="67" t="s">
+      <c r="X482" t="s">
         <v>1660</v>
       </c>
-      <c r="Y482" s="69" t="s">
+      <c r="Y482" s="36" t="s">
         <v>1661</v>
       </c>
-      <c r="Z482" s="69" t="s">
-        <v>1048</v>
-      </c>
-      <c r="AA482" s="114" t="s">
+      <c r="Z482" s="36" t="s">
+        <v>1048</v>
+      </c>
+      <c r="AA482" s="110" t="s">
         <v>1201</v>
       </c>
       <c r="AB482" s="102" t="s">
         <v>1011</v>
       </c>
-      <c r="AC482" s="67" t="s">
+      <c r="AC482" t="s">
         <v>1662</v>
       </c>
-      <c r="AD482" s="69" t="s">
+      <c r="AD482" s="36" t="s">
         <v>1663</v>
       </c>
-      <c r="AE482" s="69" t="s">
+      <c r="AE482" s="36" t="s">
         <v>1048</v>
       </c>
     </row>
     <row r="483" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A483" s="70">
-        <v>40031</v>
+        <v>40033</v>
       </c>
       <c r="B483" s="73" t="s">
-        <v>1669</v>
+        <v>1678</v>
       </c>
       <c r="C483" t="s">
         <v>1671</v>
@@ -54439,7 +54524,7 @@
         <v>2</v>
       </c>
       <c r="H483" s="73" t="s">
-        <v>1657</v>
+        <v>1675</v>
       </c>
       <c r="I483" s="73" t="s">
         <v>104</v>
@@ -54472,7 +54557,7 @@
         <v>1659</v>
       </c>
       <c r="T483" s="51" t="s">
-        <v>1657</v>
+        <v>146</v>
       </c>
       <c r="U483" s="23" t="s">
         <v>1664</v>
@@ -54508,104 +54593,104 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="484" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A484" s="70">
-        <v>40032</v>
-      </c>
-      <c r="B484" s="73" t="s">
-        <v>1677</v>
-      </c>
-      <c r="C484" t="s">
+    <row r="484" spans="1:31" s="67" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A484" s="78">
+        <v>40034</v>
+      </c>
+      <c r="B484" s="63" t="s">
+        <v>1679</v>
+      </c>
+      <c r="C484" s="67" t="s">
         <v>1670</v>
       </c>
-      <c r="D484" s="73" t="s">
+      <c r="D484" s="63" t="s">
         <v>1278</v>
       </c>
-      <c r="E484" s="73" t="s">
+      <c r="E484" s="63" t="s">
         <v>1201</v>
       </c>
-      <c r="F484" s="73" t="s">
+      <c r="F484" s="63" t="s">
         <v>1201</v>
       </c>
-      <c r="G484" s="23">
-        <v>2</v>
-      </c>
-      <c r="H484" s="73" t="s">
-        <v>1675</v>
-      </c>
-      <c r="I484" s="73" t="s">
+      <c r="G484" s="64">
+        <v>2</v>
+      </c>
+      <c r="H484" s="63" t="s">
+        <v>1656</v>
+      </c>
+      <c r="I484" s="63" t="s">
         <v>104</v>
       </c>
-      <c r="J484">
-        <v>1</v>
-      </c>
-      <c r="K484">
-        <v>1</v>
-      </c>
-      <c r="M484">
+      <c r="J484" s="67">
+        <v>1</v>
+      </c>
+      <c r="K484" s="67">
+        <v>1</v>
+      </c>
+      <c r="M484" s="67">
         <v>8</v>
       </c>
-      <c r="N484" t="s">
-        <v>1666</v>
-      </c>
-      <c r="O484" t="s">
-        <v>1667</v>
-      </c>
-      <c r="P484" s="70" t="s">
+      <c r="N484" s="67" t="s">
+        <v>1681</v>
+      </c>
+      <c r="O484" s="67" t="s">
+        <v>1683</v>
+      </c>
+      <c r="P484" s="78" t="s">
         <v>572</v>
       </c>
-      <c r="Q484" t="s">
+      <c r="Q484" s="67" t="s">
         <v>1674</v>
       </c>
-      <c r="R484" s="107" t="s">
+      <c r="R484" s="112" t="s">
         <v>1658</v>
       </c>
-      <c r="S484" t="s">
+      <c r="S484" s="67" t="s">
         <v>1659</v>
       </c>
-      <c r="T484" s="51" t="s">
-        <v>146</v>
-      </c>
-      <c r="U484" s="23" t="s">
+      <c r="T484" s="83" t="s">
+        <v>1656</v>
+      </c>
+      <c r="U484" s="64" t="s">
         <v>1001</v>
       </c>
-      <c r="V484" s="108" t="s">
+      <c r="V484" s="113" t="s">
         <v>1201</v>
       </c>
       <c r="W484" s="102" t="s">
         <v>933</v>
       </c>
-      <c r="X484" t="s">
+      <c r="X484" s="67" t="s">
         <v>1660</v>
       </c>
-      <c r="Y484" s="36" t="s">
+      <c r="Y484" s="69" t="s">
         <v>1661</v>
       </c>
-      <c r="Z484" s="36" t="s">
-        <v>1048</v>
-      </c>
-      <c r="AA484" s="110" t="s">
+      <c r="Z484" s="69" t="s">
+        <v>1048</v>
+      </c>
+      <c r="AA484" s="114" t="s">
         <v>1201</v>
       </c>
       <c r="AB484" s="102" t="s">
         <v>1011</v>
       </c>
-      <c r="AC484" t="s">
+      <c r="AC484" s="67" t="s">
         <v>1662</v>
       </c>
-      <c r="AD484" s="36" t="s">
+      <c r="AD484" s="69" t="s">
         <v>1663</v>
       </c>
-      <c r="AE484" s="36" t="s">
+      <c r="AE484" s="69" t="s">
         <v>1048</v>
       </c>
     </row>
     <row r="485" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A485" s="70">
-        <v>40033</v>
+        <v>40035</v>
       </c>
       <c r="B485" s="73" t="s">
-        <v>1678</v>
+        <v>1680</v>
       </c>
       <c r="C485" t="s">
         <v>1671</v>
@@ -54623,7 +54708,7 @@
         <v>2</v>
       </c>
       <c r="H485" s="73" t="s">
-        <v>1675</v>
+        <v>1657</v>
       </c>
       <c r="I485" s="73" t="s">
         <v>104</v>
@@ -54638,10 +54723,10 @@
         <v>8</v>
       </c>
       <c r="N485" t="s">
-        <v>1672</v>
+        <v>1682</v>
       </c>
       <c r="O485" t="s">
-        <v>1673</v>
+        <v>1684</v>
       </c>
       <c r="P485" s="70" t="s">
         <v>572</v>
@@ -54656,7 +54741,7 @@
         <v>1659</v>
       </c>
       <c r="T485" s="51" t="s">
-        <v>146</v>
+        <v>1657</v>
       </c>
       <c r="U485" s="23" t="s">
         <v>1664</v>
@@ -54692,1779 +54777,1445 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="486" spans="1:31" s="67" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="486" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A486" s="78">
-        <v>40034</v>
-      </c>
-      <c r="B486" s="63" t="s">
-        <v>1679</v>
-      </c>
-      <c r="C486" s="67" t="s">
-        <v>1670</v>
-      </c>
-      <c r="D486" s="63" t="s">
+        <v>40036</v>
+      </c>
+      <c r="B486" s="73" t="s">
+        <v>1685</v>
+      </c>
+      <c r="C486" t="s">
+        <v>1686</v>
+      </c>
+      <c r="D486" s="73" t="s">
         <v>1278</v>
       </c>
-      <c r="E486" s="63" t="s">
+      <c r="E486" s="73" t="s">
         <v>1201</v>
       </c>
-      <c r="F486" s="63" t="s">
+      <c r="F486" s="73" t="s">
         <v>1201</v>
       </c>
-      <c r="G486" s="64">
-        <v>2</v>
-      </c>
-      <c r="H486" s="63" t="s">
-        <v>1656</v>
-      </c>
-      <c r="I486" s="63" t="s">
+      <c r="G486" s="23">
+        <v>2</v>
+      </c>
+      <c r="H486" s="73" t="s">
+        <v>111</v>
+      </c>
+      <c r="I486" s="73" t="s">
         <v>104</v>
       </c>
-      <c r="J486" s="67">
-        <v>1</v>
-      </c>
-      <c r="K486" s="67">
-        <v>1</v>
-      </c>
-      <c r="M486" s="67">
+      <c r="J486">
+        <v>1</v>
+      </c>
+      <c r="K486">
+        <v>1</v>
+      </c>
+      <c r="M486">
         <v>8</v>
       </c>
-      <c r="N486" s="67" t="s">
-        <v>1681</v>
-      </c>
-      <c r="O486" s="67" t="s">
-        <v>1683</v>
-      </c>
-      <c r="P486" s="78" t="s">
+      <c r="N486" t="s">
+        <v>1695</v>
+      </c>
+      <c r="O486" t="s">
+        <v>1696</v>
+      </c>
+      <c r="P486" s="70" t="s">
         <v>572</v>
       </c>
-      <c r="Q486" s="67" t="s">
-        <v>1674</v>
-      </c>
-      <c r="R486" s="112" t="s">
-        <v>1658</v>
+      <c r="Q486" t="s">
+        <v>1697</v>
+      </c>
+      <c r="R486" s="67" t="s">
+        <v>1687</v>
       </c>
       <c r="S486" s="67" t="s">
-        <v>1659</v>
-      </c>
-      <c r="T486" s="83" t="s">
-        <v>1656</v>
-      </c>
-      <c r="U486" s="64" t="s">
-        <v>1001</v>
-      </c>
-      <c r="V486" s="113" t="s">
+        <v>1688</v>
+      </c>
+      <c r="T486" s="67" t="s">
+        <v>1689</v>
+      </c>
+      <c r="U486" s="67" t="s">
+        <v>1690</v>
+      </c>
+      <c r="V486" s="67" t="s">
         <v>1201</v>
       </c>
-      <c r="W486" s="102" t="s">
-        <v>933</v>
+      <c r="W486" s="67" t="s">
+        <v>934</v>
       </c>
       <c r="X486" s="67" t="s">
-        <v>1660</v>
-      </c>
-      <c r="Y486" s="69" t="s">
-        <v>1661</v>
-      </c>
-      <c r="Z486" s="69" t="s">
-        <v>1048</v>
-      </c>
-      <c r="AA486" s="114" t="s">
+        <v>1691</v>
+      </c>
+      <c r="Y486" s="67" t="s">
+        <v>1692</v>
+      </c>
+      <c r="Z486" s="36" t="s">
+        <v>1048</v>
+      </c>
+      <c r="AA486" s="67" t="s">
         <v>1201</v>
       </c>
-      <c r="AB486" s="102" t="s">
-        <v>1011</v>
+      <c r="AB486" s="67" t="s">
+        <v>1693</v>
       </c>
       <c r="AC486" s="67" t="s">
-        <v>1662</v>
-      </c>
-      <c r="AD486" s="69" t="s">
-        <v>1663</v>
-      </c>
-      <c r="AE486" s="69" t="s">
+        <v>1691</v>
+      </c>
+      <c r="AD486" s="67" t="s">
+        <v>1694</v>
+      </c>
+      <c r="AE486" s="36" t="s">
         <v>1048</v>
       </c>
     </row>
     <row r="487" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A487" s="70">
-        <v>40035</v>
-      </c>
-      <c r="B487" s="73" t="s">
-        <v>1680</v>
-      </c>
-      <c r="C487" t="s">
-        <v>1671</v>
-      </c>
-      <c r="D487" s="73" t="s">
-        <v>1278</v>
-      </c>
-      <c r="E487" s="73" t="s">
-        <v>1201</v>
-      </c>
-      <c r="F487" s="73" t="s">
-        <v>1201</v>
-      </c>
-      <c r="G487" s="23">
-        <v>2</v>
-      </c>
-      <c r="H487" s="73" t="s">
-        <v>1657</v>
-      </c>
-      <c r="I487" s="73" t="s">
-        <v>104</v>
-      </c>
-      <c r="J487">
-        <v>1</v>
-      </c>
-      <c r="K487">
-        <v>1</v>
-      </c>
-      <c r="M487">
-        <v>8</v>
-      </c>
-      <c r="N487" t="s">
-        <v>1682</v>
-      </c>
-      <c r="O487" t="s">
-        <v>1684</v>
-      </c>
-      <c r="P487" s="70" t="s">
-        <v>572</v>
-      </c>
-      <c r="Q487" t="s">
-        <v>1665</v>
-      </c>
-      <c r="R487" s="107" t="s">
-        <v>1658</v>
-      </c>
-      <c r="S487" t="s">
-        <v>1659</v>
-      </c>
-      <c r="T487" s="51" t="s">
-        <v>1657</v>
-      </c>
-      <c r="U487" s="23" t="s">
-        <v>1664</v>
-      </c>
-      <c r="V487" s="108" t="s">
-        <v>1201</v>
-      </c>
-      <c r="W487" s="102" t="s">
-        <v>933</v>
-      </c>
-      <c r="X487" t="s">
-        <v>1660</v>
-      </c>
-      <c r="Y487" s="36" t="s">
-        <v>1661</v>
-      </c>
-      <c r="Z487" s="36" t="s">
-        <v>1048</v>
-      </c>
-      <c r="AA487" s="110" t="s">
-        <v>1201</v>
-      </c>
-      <c r="AB487" s="102" t="s">
-        <v>1011</v>
-      </c>
-      <c r="AC487" t="s">
-        <v>1662</v>
-      </c>
-      <c r="AD487" s="36" t="s">
-        <v>1663</v>
-      </c>
-      <c r="AE487" s="36" t="s">
-        <v>1048</v>
-      </c>
-    </row>
-    <row r="488" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A488" s="78">
-        <v>40036</v>
-      </c>
-      <c r="B488" s="73" t="s">
-        <v>1685</v>
-      </c>
-      <c r="C488" t="s">
-        <v>1686</v>
-      </c>
-      <c r="D488" s="73" t="s">
-        <v>1278</v>
-      </c>
-      <c r="E488" s="73" t="s">
-        <v>1201</v>
-      </c>
-      <c r="F488" s="73" t="s">
-        <v>1201</v>
-      </c>
-      <c r="G488" s="23">
-        <v>2</v>
-      </c>
-      <c r="H488" s="73" t="s">
-        <v>111</v>
-      </c>
-      <c r="I488" s="73" t="s">
-        <v>104</v>
-      </c>
-      <c r="J488">
-        <v>1</v>
-      </c>
-      <c r="K488">
-        <v>1</v>
-      </c>
-      <c r="M488">
-        <v>8</v>
-      </c>
-      <c r="N488" t="s">
-        <v>1695</v>
-      </c>
-      <c r="O488" t="s">
-        <v>1696</v>
-      </c>
-      <c r="P488" s="70" t="s">
-        <v>572</v>
-      </c>
-      <c r="Q488" t="s">
-        <v>1697</v>
-      </c>
-      <c r="R488" s="67" t="s">
-        <v>1687</v>
-      </c>
-      <c r="S488" s="67" t="s">
-        <v>1688</v>
-      </c>
-      <c r="T488" s="67" t="s">
-        <v>1689</v>
-      </c>
-      <c r="U488" s="67" t="s">
-        <v>1690</v>
-      </c>
-      <c r="V488" s="67" t="s">
-        <v>1201</v>
-      </c>
-      <c r="W488" s="67" t="s">
-        <v>934</v>
-      </c>
-      <c r="X488" s="67" t="s">
-        <v>1691</v>
-      </c>
-      <c r="Y488" s="67" t="s">
-        <v>1692</v>
-      </c>
-      <c r="Z488" s="36" t="s">
-        <v>1048</v>
-      </c>
-      <c r="AA488" s="67" t="s">
-        <v>1201</v>
-      </c>
-      <c r="AB488" s="67" t="s">
-        <v>1693</v>
-      </c>
-      <c r="AC488" s="67" t="s">
-        <v>1691</v>
-      </c>
-      <c r="AD488" s="67" t="s">
-        <v>1694</v>
-      </c>
-      <c r="AE488" s="36" t="s">
-        <v>1048</v>
-      </c>
-    </row>
-    <row r="489" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A489" s="78">
-        <v>40037</v>
-      </c>
-      <c r="B489" s="63" t="s">
-        <v>1698</v>
-      </c>
-      <c r="C489" s="63" t="s">
-        <v>1699</v>
-      </c>
-      <c r="D489" s="73" t="s">
-        <v>1278</v>
-      </c>
-      <c r="E489" s="73" t="s">
-        <v>1201</v>
-      </c>
-      <c r="F489" s="73" t="s">
-        <v>1201</v>
-      </c>
-      <c r="G489" s="23">
-        <v>3</v>
-      </c>
-      <c r="H489" s="71" t="s">
-        <v>111</v>
-      </c>
-      <c r="I489" s="73" t="s">
-        <v>1700</v>
-      </c>
-      <c r="J489">
-        <v>1</v>
-      </c>
-      <c r="K489">
-        <v>1</v>
-      </c>
-      <c r="M489">
-        <v>8</v>
-      </c>
-      <c r="N489" t="s">
-        <v>1591</v>
-      </c>
-      <c r="O489" t="s">
-        <v>1592</v>
-      </c>
-      <c r="P489" s="38" t="s">
-        <v>572</v>
-      </c>
-      <c r="Q489" t="s">
-        <v>1586</v>
-      </c>
-      <c r="R489" s="33" t="s">
-        <v>95</v>
-      </c>
-      <c r="S489" s="62" t="s">
-        <v>784</v>
-      </c>
-      <c r="T489" s="83" t="s">
-        <v>964</v>
-      </c>
-      <c r="U489" s="67" t="s">
-        <v>1000</v>
-      </c>
-      <c r="V489" s="62" t="s">
-        <v>788</v>
-      </c>
-      <c r="W489" s="102" t="s">
-        <v>933</v>
-      </c>
-      <c r="X489" s="103" t="s">
-        <v>1038</v>
-      </c>
-      <c r="Y489" s="101" t="s">
-        <v>785</v>
-      </c>
-      <c r="Z489" s="101" t="s">
-        <v>1595</v>
-      </c>
-      <c r="AA489" s="62" t="s">
-        <v>787</v>
-      </c>
-      <c r="AB489" s="102" t="s">
-        <v>1011</v>
-      </c>
-      <c r="AC489" s="103" t="s">
-        <v>1038</v>
-      </c>
-      <c r="AD489" s="101" t="s">
-        <v>785</v>
-      </c>
-      <c r="AE489" s="101" t="s">
-        <v>1595</v>
-      </c>
-    </row>
-    <row r="490" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A490" s="78">
-        <v>40038</v>
-      </c>
-    </row>
-    <row r="491" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A491" s="70">
-        <v>40039</v>
-      </c>
-    </row>
-    <row r="492" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A492" s="78">
-        <v>40040</v>
-      </c>
-    </row>
-    <row r="493" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A493" s="70">
-        <v>40041</v>
-      </c>
-    </row>
-    <row r="494" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A494" s="78">
-        <v>40042</v>
-      </c>
-    </row>
-    <row r="495" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A495" s="70">
-        <v>40043</v>
-      </c>
-    </row>
-    <row r="496" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A496" s="78">
-        <v>40044</v>
-      </c>
-    </row>
-    <row r="497" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A497" s="70">
-        <v>40045</v>
-      </c>
+      <c r="A487" s="70"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="I1:I163 I166 I267:I303 I314 I309:I311 I306 I317 I323 I327:I328 I325 I169:I265 I431:I442 I446 I331:I338 I319 I321 I367 I369 I371:I429 I356 I359 I362:I365 I341 I344 I347:I353">
-    <cfRule type="containsText" dxfId="361" priority="491" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="356" priority="491" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I1)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="360" priority="492" operator="equal">
+    <cfRule type="cellIs" dxfId="355" priority="492" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="359" priority="493" operator="equal">
+    <cfRule type="cellIs" dxfId="354" priority="493" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="358" priority="494" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="353" priority="494" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I189:I194">
-    <cfRule type="containsText" dxfId="357" priority="443" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="352" priority="443" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I189)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="356" priority="444" operator="equal">
+    <cfRule type="cellIs" dxfId="351" priority="444" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="355" priority="445" operator="equal">
+    <cfRule type="cellIs" dxfId="350" priority="445" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="354" priority="446" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="349" priority="446" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I189)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I195:I200">
-    <cfRule type="containsText" dxfId="353" priority="439" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="348" priority="439" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I195)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="352" priority="440" operator="equal">
+    <cfRule type="cellIs" dxfId="347" priority="440" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="351" priority="441" operator="equal">
+    <cfRule type="cellIs" dxfId="346" priority="441" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="350" priority="442" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="345" priority="442" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I195)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I207">
-    <cfRule type="containsText" dxfId="349" priority="435" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="344" priority="435" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I207)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="348" priority="436" operator="equal">
+    <cfRule type="cellIs" dxfId="343" priority="436" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="347" priority="437" operator="equal">
+    <cfRule type="cellIs" dxfId="342" priority="437" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="346" priority="438" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="341" priority="438" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I207)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I214">
-    <cfRule type="containsText" dxfId="345" priority="431" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="340" priority="431" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I214)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="344" priority="432" operator="equal">
+    <cfRule type="cellIs" dxfId="339" priority="432" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="343" priority="433" operator="equal">
+    <cfRule type="cellIs" dxfId="338" priority="433" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="342" priority="434" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="337" priority="434" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I214)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I221">
-    <cfRule type="containsText" dxfId="341" priority="427" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="336" priority="427" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I221)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="340" priority="428" operator="equal">
+    <cfRule type="cellIs" dxfId="335" priority="428" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="339" priority="429" operator="equal">
+    <cfRule type="cellIs" dxfId="334" priority="429" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="338" priority="430" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="333" priority="430" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I221)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I229:I234">
-    <cfRule type="containsText" dxfId="337" priority="423" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="332" priority="423" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I229)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="336" priority="424" operator="equal">
+    <cfRule type="cellIs" dxfId="331" priority="424" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="335" priority="425" operator="equal">
+    <cfRule type="cellIs" dxfId="330" priority="425" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="334" priority="426" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="329" priority="426" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I229)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I228">
-    <cfRule type="containsText" dxfId="333" priority="419" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="328" priority="419" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I228)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="332" priority="420" operator="equal">
+    <cfRule type="cellIs" dxfId="327" priority="420" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="331" priority="421" operator="equal">
+    <cfRule type="cellIs" dxfId="326" priority="421" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="330" priority="422" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="325" priority="422" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I228)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I235">
-    <cfRule type="containsText" dxfId="329" priority="415" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="324" priority="415" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I235)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="328" priority="416" operator="equal">
+    <cfRule type="cellIs" dxfId="323" priority="416" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="327" priority="417" operator="equal">
+    <cfRule type="cellIs" dxfId="322" priority="417" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="326" priority="418" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="321" priority="418" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I235)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I236:I241">
-    <cfRule type="containsText" dxfId="325" priority="411" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="320" priority="411" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I236)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="324" priority="412" operator="equal">
+    <cfRule type="cellIs" dxfId="319" priority="412" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="323" priority="413" operator="equal">
+    <cfRule type="cellIs" dxfId="318" priority="413" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="322" priority="414" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="317" priority="414" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I236)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I242">
-    <cfRule type="containsText" dxfId="321" priority="407" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="316" priority="407" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I242)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="320" priority="408" operator="equal">
+    <cfRule type="cellIs" dxfId="315" priority="408" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="319" priority="409" operator="equal">
+    <cfRule type="cellIs" dxfId="314" priority="409" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="318" priority="410" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="313" priority="410" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I242)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I164">
-    <cfRule type="containsText" dxfId="317" priority="395" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="312" priority="395" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I164)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="316" priority="396" operator="equal">
+    <cfRule type="cellIs" dxfId="311" priority="396" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="315" priority="397" operator="equal">
+    <cfRule type="cellIs" dxfId="310" priority="397" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="314" priority="398" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="309" priority="398" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I164)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I165">
-    <cfRule type="containsText" dxfId="313" priority="391" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="308" priority="391" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I165)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="312" priority="392" operator="equal">
+    <cfRule type="cellIs" dxfId="307" priority="392" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="311" priority="393" operator="equal">
+    <cfRule type="cellIs" dxfId="306" priority="393" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="310" priority="394" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="305" priority="394" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I165)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I168">
-    <cfRule type="containsText" dxfId="309" priority="387" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="304" priority="387" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I168)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="308" priority="388" operator="equal">
+    <cfRule type="cellIs" dxfId="303" priority="388" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="307" priority="389" operator="equal">
+    <cfRule type="cellIs" dxfId="302" priority="389" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="306" priority="390" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="301" priority="390" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I168)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I167">
-    <cfRule type="containsText" dxfId="305" priority="383" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="300" priority="383" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I167)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="304" priority="384" operator="equal">
+    <cfRule type="cellIs" dxfId="299" priority="384" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="303" priority="385" operator="equal">
+    <cfRule type="cellIs" dxfId="298" priority="385" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="302" priority="386" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="297" priority="386" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I167)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I266">
-    <cfRule type="containsText" dxfId="301" priority="375" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="296" priority="375" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I266)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="300" priority="376" operator="equal">
+    <cfRule type="cellIs" dxfId="295" priority="376" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="299" priority="377" operator="equal">
+    <cfRule type="cellIs" dxfId="294" priority="377" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="298" priority="378" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="293" priority="378" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I266)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I313">
-    <cfRule type="containsText" dxfId="297" priority="371" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="292" priority="371" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I313)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="296" priority="372" operator="equal">
+    <cfRule type="cellIs" dxfId="291" priority="372" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="295" priority="373" operator="equal">
+    <cfRule type="cellIs" dxfId="290" priority="373" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="294" priority="374" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="289" priority="374" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I313)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I316">
-    <cfRule type="containsText" dxfId="293" priority="367" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="288" priority="367" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I316)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="292" priority="368" operator="equal">
+    <cfRule type="cellIs" dxfId="287" priority="368" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="291" priority="369" operator="equal">
+    <cfRule type="cellIs" dxfId="286" priority="369" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="290" priority="370" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="285" priority="370" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I316)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I307">
-    <cfRule type="containsText" dxfId="289" priority="363" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="284" priority="363" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I307)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="288" priority="364" operator="equal">
+    <cfRule type="cellIs" dxfId="283" priority="364" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="287" priority="365" operator="equal">
+    <cfRule type="cellIs" dxfId="282" priority="365" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="286" priority="366" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="281" priority="366" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I307)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I304">
-    <cfRule type="containsText" dxfId="285" priority="359" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="280" priority="359" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I304)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="284" priority="360" operator="equal">
+    <cfRule type="cellIs" dxfId="279" priority="360" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="283" priority="361" operator="equal">
+    <cfRule type="cellIs" dxfId="278" priority="361" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="282" priority="362" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="277" priority="362" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I304)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I305">
-    <cfRule type="containsText" dxfId="281" priority="355" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="276" priority="355" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I305)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="280" priority="356" operator="equal">
+    <cfRule type="cellIs" dxfId="275" priority="356" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="279" priority="357" operator="equal">
+    <cfRule type="cellIs" dxfId="274" priority="357" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="278" priority="358" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="273" priority="358" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I305)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I308">
-    <cfRule type="containsText" dxfId="277" priority="351" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="272" priority="351" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I308)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="276" priority="352" operator="equal">
+    <cfRule type="cellIs" dxfId="271" priority="352" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="275" priority="353" operator="equal">
+    <cfRule type="cellIs" dxfId="270" priority="353" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="274" priority="354" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="269" priority="354" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I308)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I322">
-    <cfRule type="containsText" dxfId="273" priority="347" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="268" priority="347" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I322)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="272" priority="348" operator="equal">
+    <cfRule type="cellIs" dxfId="267" priority="348" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="271" priority="349" operator="equal">
+    <cfRule type="cellIs" dxfId="266" priority="349" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="270" priority="350" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="265" priority="350" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I322)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I326">
-    <cfRule type="containsText" dxfId="269" priority="343" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="264" priority="343" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I326)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="268" priority="344" operator="equal">
+    <cfRule type="cellIs" dxfId="263" priority="344" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="267" priority="345" operator="equal">
+    <cfRule type="cellIs" dxfId="262" priority="345" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="266" priority="346" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="261" priority="346" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I326)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I324">
-    <cfRule type="containsText" dxfId="265" priority="339" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="260" priority="339" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I324)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="264" priority="340" operator="equal">
+    <cfRule type="cellIs" dxfId="259" priority="340" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="263" priority="341" operator="equal">
+    <cfRule type="cellIs" dxfId="258" priority="341" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="262" priority="342" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="257" priority="342" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I324)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E1:F2 E313:E314 E316:E317 E319 E321:E328 E331:E338 E3:E311 F3:F338 E367:F367 E369:F369 E371:F446 E356:F356 E359:F359 E362:F365 E341:F341 E344:F344 E347:F353 E453:F463 E481:F483 E490:F1048576">
-    <cfRule type="cellIs" dxfId="261" priority="337" operator="equal">
+  <conditionalFormatting sqref="E1:F2 E313:E314 E316:E317 E319 E321:E328 E331:E338 E3:E311 F3:F338 E367:F367 E369:F369 E371:F446 E356:F356 E359:F359 E362:F365 E341:F341 E344:F344 E347:F353 E479:F481 E487:F1048576 E453:F461">
+    <cfRule type="cellIs" dxfId="256" priority="337" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="260" priority="338" operator="equal">
+    <cfRule type="cellIs" dxfId="255" priority="338" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I329:I330">
-    <cfRule type="containsText" dxfId="259" priority="333" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="254" priority="333" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I329)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="258" priority="334" operator="equal">
+    <cfRule type="cellIs" dxfId="253" priority="334" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="257" priority="335" operator="equal">
+    <cfRule type="cellIs" dxfId="252" priority="335" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="256" priority="336" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="251" priority="336" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I329)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E329:E330">
-    <cfRule type="cellIs" dxfId="255" priority="331" operator="equal">
+    <cfRule type="cellIs" dxfId="250" priority="331" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="254" priority="332" operator="equal">
+    <cfRule type="cellIs" dxfId="249" priority="332" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I430">
-    <cfRule type="containsText" dxfId="253" priority="321" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="248" priority="321" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I430)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="252" priority="322" operator="equal">
+    <cfRule type="cellIs" dxfId="247" priority="322" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="251" priority="323" operator="equal">
+    <cfRule type="cellIs" dxfId="246" priority="323" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="250" priority="324" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="245" priority="324" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I430)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E430:F430">
-    <cfRule type="cellIs" dxfId="249" priority="319" operator="equal">
+    <cfRule type="cellIs" dxfId="244" priority="319" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="248" priority="320" operator="equal">
+    <cfRule type="cellIs" dxfId="243" priority="320" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I443">
-    <cfRule type="containsText" dxfId="247" priority="315" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="242" priority="315" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I443)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="246" priority="316" operator="equal">
+    <cfRule type="cellIs" dxfId="241" priority="316" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="245" priority="317" operator="equal">
+    <cfRule type="cellIs" dxfId="240" priority="317" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="244" priority="318" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="239" priority="318" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I443)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E443:F443">
-    <cfRule type="cellIs" dxfId="243" priority="313" operator="equal">
+    <cfRule type="cellIs" dxfId="238" priority="313" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="242" priority="314" operator="equal">
+    <cfRule type="cellIs" dxfId="237" priority="314" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I444">
-    <cfRule type="containsText" dxfId="241" priority="309" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="236" priority="309" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I444)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="240" priority="310" operator="equal">
+    <cfRule type="cellIs" dxfId="235" priority="310" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="239" priority="311" operator="equal">
+    <cfRule type="cellIs" dxfId="234" priority="311" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="238" priority="312" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="233" priority="312" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I444)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E444:F444">
-    <cfRule type="cellIs" dxfId="237" priority="307" operator="equal">
+    <cfRule type="cellIs" dxfId="232" priority="307" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="236" priority="308" operator="equal">
+    <cfRule type="cellIs" dxfId="231" priority="308" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I445">
-    <cfRule type="containsText" dxfId="235" priority="303" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="230" priority="303" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I445)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="234" priority="304" operator="equal">
+    <cfRule type="cellIs" dxfId="229" priority="304" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="233" priority="305" operator="equal">
+    <cfRule type="cellIs" dxfId="228" priority="305" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="232" priority="306" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="227" priority="306" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I445)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E445:F445">
-    <cfRule type="cellIs" dxfId="231" priority="301" operator="equal">
+    <cfRule type="cellIs" dxfId="226" priority="301" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="230" priority="302" operator="equal">
+    <cfRule type="cellIs" dxfId="225" priority="302" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E1:F2 E313:E314 E316:E317 E319 E321:E338 E3:E311 F3:F338 E367:F367 E369:F369 E371:F446 E356:F356 E359:F359 E362:F365 E341:F341 E344:F344 E347:F353 E453:F463 E481:F483 E490:F1048576">
-    <cfRule type="cellIs" dxfId="229" priority="300" operator="equal">
+  <conditionalFormatting sqref="E1:F2 E313:E314 E316:E317 E319 E321:E338 E3:E311 F3:F338 E367:F367 E369:F369 E371:F446 E356:F356 E359:F359 E362:F365 E341:F341 E344:F344 E347:F353 E479:F481 E487:F1048576 E453:F461">
+    <cfRule type="cellIs" dxfId="224" priority="300" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I312">
-    <cfRule type="containsText" dxfId="228" priority="268" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="223" priority="268" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I312)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="227" priority="269" operator="equal">
+    <cfRule type="cellIs" dxfId="222" priority="269" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="226" priority="270" operator="equal">
+    <cfRule type="cellIs" dxfId="221" priority="270" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="225" priority="271" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="220" priority="271" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I312)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E312">
-    <cfRule type="cellIs" dxfId="224" priority="266" operator="equal">
+    <cfRule type="cellIs" dxfId="219" priority="266" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="223" priority="267" operator="equal">
+    <cfRule type="cellIs" dxfId="218" priority="267" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E312">
-    <cfRule type="cellIs" dxfId="222" priority="265" operator="equal">
+    <cfRule type="cellIs" dxfId="217" priority="265" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I315">
-    <cfRule type="containsText" dxfId="221" priority="261" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="216" priority="261" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I315)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="220" priority="262" operator="equal">
+    <cfRule type="cellIs" dxfId="215" priority="262" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="219" priority="263" operator="equal">
+    <cfRule type="cellIs" dxfId="214" priority="263" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="218" priority="264" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="213" priority="264" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I315)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E315">
-    <cfRule type="cellIs" dxfId="217" priority="259" operator="equal">
+    <cfRule type="cellIs" dxfId="212" priority="259" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="216" priority="260" operator="equal">
+    <cfRule type="cellIs" dxfId="211" priority="260" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E315">
-    <cfRule type="cellIs" dxfId="215" priority="258" operator="equal">
+    <cfRule type="cellIs" dxfId="210" priority="258" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I318">
-    <cfRule type="containsText" dxfId="214" priority="254" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="209" priority="254" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I318)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="213" priority="255" operator="equal">
+    <cfRule type="cellIs" dxfId="208" priority="255" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="212" priority="256" operator="equal">
+    <cfRule type="cellIs" dxfId="207" priority="256" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="211" priority="257" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="206" priority="257" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I318)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E318">
-    <cfRule type="cellIs" dxfId="210" priority="252" operator="equal">
+    <cfRule type="cellIs" dxfId="205" priority="252" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="209" priority="253" operator="equal">
+    <cfRule type="cellIs" dxfId="204" priority="253" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E318">
-    <cfRule type="cellIs" dxfId="208" priority="251" operator="equal">
+    <cfRule type="cellIs" dxfId="203" priority="251" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I320">
-    <cfRule type="containsText" dxfId="207" priority="247" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="202" priority="247" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I320)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="206" priority="248" operator="equal">
+    <cfRule type="cellIs" dxfId="201" priority="248" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="205" priority="249" operator="equal">
+    <cfRule type="cellIs" dxfId="200" priority="249" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="204" priority="250" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="199" priority="250" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I320)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E320">
-    <cfRule type="cellIs" dxfId="203" priority="245" operator="equal">
+    <cfRule type="cellIs" dxfId="198" priority="245" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="202" priority="246" operator="equal">
+    <cfRule type="cellIs" dxfId="197" priority="246" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E320">
-    <cfRule type="cellIs" dxfId="201" priority="244" operator="equal">
+    <cfRule type="cellIs" dxfId="196" priority="244" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F1:F338 F367 F369 F371:F446 F356 F359 F362:F365 F341 F344 F347:F353 F453:F463 F481:F483 F490:F1048576">
-    <cfRule type="cellIs" dxfId="200" priority="242" operator="equal">
+  <conditionalFormatting sqref="F1:F338 F367 F369 F371:F446 F356 F359 F362:F365 F341 F344 F347:F353 F479:F481 F487:F1048576 F453:F461">
+    <cfRule type="cellIs" dxfId="195" priority="242" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="199" priority="243" operator="equal">
+    <cfRule type="cellIs" dxfId="194" priority="243" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I447">
-    <cfRule type="containsText" dxfId="198" priority="238" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="193" priority="238" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I447)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="197" priority="239" operator="equal">
+    <cfRule type="cellIs" dxfId="192" priority="239" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="196" priority="240" operator="equal">
+    <cfRule type="cellIs" dxfId="191" priority="240" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="195" priority="241" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="190" priority="241" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I447)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E447:F447">
-    <cfRule type="cellIs" dxfId="194" priority="236" operator="equal">
+    <cfRule type="cellIs" dxfId="189" priority="236" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="193" priority="237" operator="equal">
+    <cfRule type="cellIs" dxfId="188" priority="237" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E447:F447">
-    <cfRule type="cellIs" dxfId="192" priority="235" operator="equal">
+    <cfRule type="cellIs" dxfId="187" priority="235" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F447">
-    <cfRule type="cellIs" dxfId="191" priority="233" operator="equal">
+    <cfRule type="cellIs" dxfId="186" priority="233" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="190" priority="234" operator="equal">
+    <cfRule type="cellIs" dxfId="185" priority="234" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I448">
-    <cfRule type="containsText" dxfId="189" priority="229" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="184" priority="229" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I448)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="188" priority="230" operator="equal">
+    <cfRule type="cellIs" dxfId="183" priority="230" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="187" priority="231" operator="equal">
+    <cfRule type="cellIs" dxfId="182" priority="231" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="186" priority="232" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="181" priority="232" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I448)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E448:F448">
-    <cfRule type="cellIs" dxfId="185" priority="227" operator="equal">
+    <cfRule type="cellIs" dxfId="180" priority="227" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="184" priority="228" operator="equal">
+    <cfRule type="cellIs" dxfId="179" priority="228" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E448:F448">
-    <cfRule type="cellIs" dxfId="183" priority="226" operator="equal">
+    <cfRule type="cellIs" dxfId="178" priority="226" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F448">
-    <cfRule type="cellIs" dxfId="182" priority="224" operator="equal">
+    <cfRule type="cellIs" dxfId="177" priority="224" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="181" priority="225" operator="equal">
+    <cfRule type="cellIs" dxfId="176" priority="225" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I449">
-    <cfRule type="containsText" dxfId="180" priority="220" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="175" priority="220" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I449)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="179" priority="221" operator="equal">
+    <cfRule type="cellIs" dxfId="174" priority="221" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="178" priority="222" operator="equal">
+    <cfRule type="cellIs" dxfId="173" priority="222" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="177" priority="223" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="172" priority="223" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I449)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E449:F452">
-    <cfRule type="cellIs" dxfId="176" priority="218" operator="equal">
+    <cfRule type="cellIs" dxfId="171" priority="218" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="175" priority="219" operator="equal">
+    <cfRule type="cellIs" dxfId="170" priority="219" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E449:F452">
-    <cfRule type="cellIs" dxfId="174" priority="217" operator="equal">
+    <cfRule type="cellIs" dxfId="169" priority="217" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F449:F452">
-    <cfRule type="cellIs" dxfId="173" priority="215" operator="equal">
+    <cfRule type="cellIs" dxfId="168" priority="215" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="172" priority="216" operator="equal">
+    <cfRule type="cellIs" dxfId="167" priority="216" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I450">
-    <cfRule type="containsText" dxfId="171" priority="184" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="166" priority="184" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I450)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="170" priority="185" operator="equal">
+    <cfRule type="cellIs" dxfId="165" priority="185" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="169" priority="186" operator="equal">
+    <cfRule type="cellIs" dxfId="164" priority="186" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="168" priority="187" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="163" priority="187" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I450)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E366:F366">
-    <cfRule type="cellIs" dxfId="167" priority="155" operator="equal">
+    <cfRule type="cellIs" dxfId="162" priority="155" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="166" priority="156" operator="equal">
+    <cfRule type="cellIs" dxfId="161" priority="156" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E366:F366">
-    <cfRule type="cellIs" dxfId="165" priority="154" operator="equal">
+    <cfRule type="cellIs" dxfId="160" priority="154" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F366">
-    <cfRule type="cellIs" dxfId="164" priority="152" operator="equal">
+    <cfRule type="cellIs" dxfId="159" priority="152" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="163" priority="153" operator="equal">
+    <cfRule type="cellIs" dxfId="158" priority="153" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I451">
-    <cfRule type="containsText" dxfId="162" priority="175" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="157" priority="175" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I451)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="161" priority="176" operator="equal">
+    <cfRule type="cellIs" dxfId="156" priority="176" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="160" priority="177" operator="equal">
+    <cfRule type="cellIs" dxfId="155" priority="177" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="159" priority="178" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="154" priority="178" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I451)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E354:F354">
-    <cfRule type="cellIs" dxfId="158" priority="128" operator="equal">
+    <cfRule type="cellIs" dxfId="153" priority="128" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="157" priority="129" operator="equal">
+    <cfRule type="cellIs" dxfId="152" priority="129" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E354:F354">
-    <cfRule type="cellIs" dxfId="156" priority="127" operator="equal">
+    <cfRule type="cellIs" dxfId="151" priority="127" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F354">
-    <cfRule type="cellIs" dxfId="155" priority="125" operator="equal">
+    <cfRule type="cellIs" dxfId="150" priority="125" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="154" priority="126" operator="equal">
+    <cfRule type="cellIs" dxfId="149" priority="126" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I366">
-    <cfRule type="containsText" dxfId="153" priority="157" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="148" priority="157" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I366)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="152" priority="158" operator="equal">
+    <cfRule type="cellIs" dxfId="147" priority="158" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="151" priority="159" operator="equal">
+    <cfRule type="cellIs" dxfId="146" priority="159" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="150" priority="160" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="145" priority="160" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I366)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I354">
-    <cfRule type="containsText" dxfId="149" priority="130" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="144" priority="130" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I354)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="148" priority="131" operator="equal">
+    <cfRule type="cellIs" dxfId="143" priority="131" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="147" priority="132" operator="equal">
+    <cfRule type="cellIs" dxfId="142" priority="132" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="146" priority="133" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="141" priority="133" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I354)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E368:F368">
-    <cfRule type="cellIs" dxfId="145" priority="146" operator="equal">
+    <cfRule type="cellIs" dxfId="140" priority="146" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="144" priority="147" operator="equal">
+    <cfRule type="cellIs" dxfId="139" priority="147" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E368:F368">
-    <cfRule type="cellIs" dxfId="143" priority="145" operator="equal">
+    <cfRule type="cellIs" dxfId="138" priority="145" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F368">
-    <cfRule type="cellIs" dxfId="142" priority="143" operator="equal">
+    <cfRule type="cellIs" dxfId="137" priority="143" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="141" priority="144" operator="equal">
+    <cfRule type="cellIs" dxfId="136" priority="144" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I452">
-    <cfRule type="containsText" dxfId="140" priority="166" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="135" priority="166" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I452)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="139" priority="167" operator="equal">
+    <cfRule type="cellIs" dxfId="134" priority="167" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="138" priority="168" operator="equal">
+    <cfRule type="cellIs" dxfId="133" priority="168" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="137" priority="169" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="132" priority="169" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I452)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E370:F370">
-    <cfRule type="cellIs" dxfId="136" priority="137" operator="equal">
+    <cfRule type="cellIs" dxfId="131" priority="137" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="135" priority="138" operator="equal">
+    <cfRule type="cellIs" dxfId="130" priority="138" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E370:F370">
-    <cfRule type="cellIs" dxfId="134" priority="136" operator="equal">
+    <cfRule type="cellIs" dxfId="129" priority="136" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F370">
-    <cfRule type="cellIs" dxfId="133" priority="134" operator="equal">
+    <cfRule type="cellIs" dxfId="128" priority="134" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="132" priority="135" operator="equal">
+    <cfRule type="cellIs" dxfId="127" priority="135" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I368">
-    <cfRule type="containsText" dxfId="131" priority="148" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="126" priority="148" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I368)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="130" priority="149" operator="equal">
+    <cfRule type="cellIs" dxfId="125" priority="149" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="129" priority="150" operator="equal">
+    <cfRule type="cellIs" dxfId="124" priority="150" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="128" priority="151" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="123" priority="151" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I368)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E357:F357">
-    <cfRule type="cellIs" dxfId="127" priority="119" operator="equal">
+    <cfRule type="cellIs" dxfId="122" priority="119" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="126" priority="120" operator="equal">
+    <cfRule type="cellIs" dxfId="121" priority="120" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E357:F357">
-    <cfRule type="cellIs" dxfId="125" priority="118" operator="equal">
+    <cfRule type="cellIs" dxfId="120" priority="118" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F357">
-    <cfRule type="cellIs" dxfId="124" priority="116" operator="equal">
+    <cfRule type="cellIs" dxfId="119" priority="116" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="123" priority="117" operator="equal">
+    <cfRule type="cellIs" dxfId="118" priority="117" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I370">
-    <cfRule type="containsText" dxfId="122" priority="139" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="117" priority="139" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I370)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="121" priority="140" operator="equal">
+    <cfRule type="cellIs" dxfId="116" priority="140" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="120" priority="141" operator="equal">
+    <cfRule type="cellIs" dxfId="115" priority="141" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="119" priority="142" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="114" priority="142" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I370)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E360:F360">
-    <cfRule type="cellIs" dxfId="118" priority="110" operator="equal">
+    <cfRule type="cellIs" dxfId="113" priority="110" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="117" priority="111" operator="equal">
+    <cfRule type="cellIs" dxfId="112" priority="111" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E360:F360">
-    <cfRule type="cellIs" dxfId="116" priority="109" operator="equal">
+    <cfRule type="cellIs" dxfId="111" priority="109" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F360">
-    <cfRule type="cellIs" dxfId="115" priority="107" operator="equal">
+    <cfRule type="cellIs" dxfId="110" priority="107" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="114" priority="108" operator="equal">
+    <cfRule type="cellIs" dxfId="109" priority="108" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I357">
-    <cfRule type="containsText" dxfId="113" priority="121" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="108" priority="121" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I357)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="112" priority="122" operator="equal">
+    <cfRule type="cellIs" dxfId="107" priority="122" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="111" priority="123" operator="equal">
+    <cfRule type="cellIs" dxfId="106" priority="123" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="110" priority="124" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="105" priority="124" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I357)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I360">
-    <cfRule type="containsText" dxfId="109" priority="112" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="104" priority="112" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I360)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="108" priority="113" operator="equal">
+    <cfRule type="cellIs" dxfId="103" priority="113" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="107" priority="114" operator="equal">
+    <cfRule type="cellIs" dxfId="102" priority="114" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="106" priority="115" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="101" priority="115" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I360)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I339">
-    <cfRule type="containsText" dxfId="105" priority="103" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="100" priority="103" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I339)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="104" priority="104" operator="equal">
+    <cfRule type="cellIs" dxfId="99" priority="104" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="103" priority="105" operator="equal">
+    <cfRule type="cellIs" dxfId="98" priority="105" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="102" priority="106" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="97" priority="106" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I339)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E339:F339">
-    <cfRule type="cellIs" dxfId="101" priority="101" operator="equal">
+    <cfRule type="cellIs" dxfId="96" priority="101" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="100" priority="102" operator="equal">
+    <cfRule type="cellIs" dxfId="95" priority="102" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E339:F339">
-    <cfRule type="cellIs" dxfId="99" priority="100" operator="equal">
+    <cfRule type="cellIs" dxfId="94" priority="100" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F339">
-    <cfRule type="cellIs" dxfId="98" priority="98" operator="equal">
+    <cfRule type="cellIs" dxfId="93" priority="98" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="97" priority="99" operator="equal">
+    <cfRule type="cellIs" dxfId="92" priority="99" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I342">
-    <cfRule type="containsText" dxfId="96" priority="94" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="91" priority="94" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I342)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="95" priority="95" operator="equal">
+    <cfRule type="cellIs" dxfId="90" priority="95" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="94" priority="96" operator="equal">
+    <cfRule type="cellIs" dxfId="89" priority="96" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="93" priority="97" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="88" priority="97" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I342)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E342:F342">
-    <cfRule type="cellIs" dxfId="92" priority="92" operator="equal">
+    <cfRule type="cellIs" dxfId="87" priority="92" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="91" priority="93" operator="equal">
+    <cfRule type="cellIs" dxfId="86" priority="93" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E342:F342">
-    <cfRule type="cellIs" dxfId="90" priority="91" operator="equal">
+    <cfRule type="cellIs" dxfId="85" priority="91" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F342">
-    <cfRule type="cellIs" dxfId="89" priority="89" operator="equal">
+    <cfRule type="cellIs" dxfId="84" priority="89" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="88" priority="90" operator="equal">
+    <cfRule type="cellIs" dxfId="83" priority="90" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I345">
-    <cfRule type="containsText" dxfId="87" priority="85" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="82" priority="85" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I345)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="86" priority="86" operator="equal">
+    <cfRule type="cellIs" dxfId="81" priority="86" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="85" priority="87" operator="equal">
+    <cfRule type="cellIs" dxfId="80" priority="87" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="84" priority="88" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="79" priority="88" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I345)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E345:F345">
-    <cfRule type="cellIs" dxfId="83" priority="83" operator="equal">
+    <cfRule type="cellIs" dxfId="78" priority="83" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="82" priority="84" operator="equal">
+    <cfRule type="cellIs" dxfId="77" priority="84" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E345:F345">
-    <cfRule type="cellIs" dxfId="81" priority="82" operator="equal">
+    <cfRule type="cellIs" dxfId="76" priority="82" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F345">
-    <cfRule type="cellIs" dxfId="80" priority="80" operator="equal">
+    <cfRule type="cellIs" dxfId="75" priority="80" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="79" priority="81" operator="equal">
+    <cfRule type="cellIs" dxfId="74" priority="81" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E355:F355">
-    <cfRule type="cellIs" dxfId="78" priority="74" operator="equal">
+    <cfRule type="cellIs" dxfId="73" priority="74" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="77" priority="75" operator="equal">
+    <cfRule type="cellIs" dxfId="72" priority="75" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E355:F355">
-    <cfRule type="cellIs" dxfId="76" priority="73" operator="equal">
+    <cfRule type="cellIs" dxfId="71" priority="73" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F355">
-    <cfRule type="cellIs" dxfId="75" priority="71" operator="equal">
+    <cfRule type="cellIs" dxfId="70" priority="71" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="74" priority="72" operator="equal">
+    <cfRule type="cellIs" dxfId="69" priority="72" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I355">
-    <cfRule type="containsText" dxfId="73" priority="76" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="68" priority="76" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I355)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="72" priority="77" operator="equal">
+    <cfRule type="cellIs" dxfId="67" priority="77" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="71" priority="78" operator="equal">
+    <cfRule type="cellIs" dxfId="66" priority="78" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="70" priority="79" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="65" priority="79" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I355)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E358:F358">
-    <cfRule type="cellIs" dxfId="69" priority="65" operator="equal">
+    <cfRule type="cellIs" dxfId="64" priority="65" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="68" priority="66" operator="equal">
+    <cfRule type="cellIs" dxfId="63" priority="66" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E358:F358">
-    <cfRule type="cellIs" dxfId="67" priority="64" operator="equal">
+    <cfRule type="cellIs" dxfId="62" priority="64" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F358">
-    <cfRule type="cellIs" dxfId="66" priority="62" operator="equal">
+    <cfRule type="cellIs" dxfId="61" priority="62" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="65" priority="63" operator="equal">
+    <cfRule type="cellIs" dxfId="60" priority="63" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I358">
-    <cfRule type="containsText" dxfId="64" priority="67" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="59" priority="67" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I358)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="63" priority="68" operator="equal">
+    <cfRule type="cellIs" dxfId="58" priority="68" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="62" priority="69" operator="equal">
+    <cfRule type="cellIs" dxfId="57" priority="69" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="61" priority="70" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="56" priority="70" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I358)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E361:F361">
-    <cfRule type="cellIs" dxfId="60" priority="56" operator="equal">
+    <cfRule type="cellIs" dxfId="55" priority="56" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="59" priority="57" operator="equal">
+    <cfRule type="cellIs" dxfId="54" priority="57" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E361:F361">
-    <cfRule type="cellIs" dxfId="58" priority="55" operator="equal">
+    <cfRule type="cellIs" dxfId="53" priority="55" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F361">
-    <cfRule type="cellIs" dxfId="57" priority="53" operator="equal">
+    <cfRule type="cellIs" dxfId="52" priority="53" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="54" operator="equal">
+    <cfRule type="cellIs" dxfId="51" priority="54" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I361">
-    <cfRule type="containsText" dxfId="55" priority="58" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="50" priority="58" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I361)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="59" operator="equal">
+    <cfRule type="cellIs" dxfId="49" priority="59" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="53" priority="60" operator="equal">
+    <cfRule type="cellIs" dxfId="48" priority="60" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="52" priority="61" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="47" priority="61" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I361)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I340">
-    <cfRule type="containsText" dxfId="51" priority="49" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="46" priority="49" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I340)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="50" operator="equal">
+    <cfRule type="cellIs" dxfId="45" priority="50" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="51" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="51" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="48" priority="52" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="43" priority="52" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I340)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E340:F340">
-    <cfRule type="cellIs" dxfId="47" priority="47" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="47" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="48" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="48" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E340:F340">
-    <cfRule type="cellIs" dxfId="45" priority="46" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="46" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F340">
-    <cfRule type="cellIs" dxfId="44" priority="44" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="44" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="45" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="45" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I343">
-    <cfRule type="containsText" dxfId="42" priority="40" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="37" priority="40" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I343)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="41" priority="41" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="41" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="42" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="42" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="39" priority="43" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="34" priority="43" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I343)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E343:F343">
-    <cfRule type="cellIs" dxfId="38" priority="38" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="38" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="39" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="39" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E343:F343">
-    <cfRule type="cellIs" dxfId="36" priority="37" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="37" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F343">
-    <cfRule type="cellIs" dxfId="35" priority="35" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="35" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="36" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="36" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I346">
-    <cfRule type="containsText" dxfId="33" priority="31" operator="containsText" text="iso">
+    <cfRule type="containsText" dxfId="28" priority="31" operator="containsText" text="iso">
       <formula>NOT(ISERROR(SEARCH("iso",I346)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="32" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="32" operator="equal">
       <formula>"dn"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="33" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="33" operator="equal">
       <formula>"dcv"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="30" priority="34" operator="containsText" text="sr">
+    <cfRule type="containsText" dxfId="25" priority="34" operator="containsText" text="sr">
       <formula>NOT(ISERROR(SEARCH("sr",I346)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E346:F346">
-    <cfRule type="cellIs" dxfId="29" priority="29" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="29" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="30" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="30" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E346:F346">
-    <cfRule type="cellIs" dxfId="27" priority="28" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="28" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F346">
-    <cfRule type="cellIs" dxfId="26" priority="26" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="26" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="27" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="27" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E464:F467">
-    <cfRule type="cellIs" dxfId="24" priority="24" operator="equal">
+  <conditionalFormatting sqref="E462:F465">
+    <cfRule type="cellIs" dxfId="19" priority="24" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="23" priority="25" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="25" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E464:F467">
-    <cfRule type="cellIs" dxfId="22" priority="23" operator="equal">
+  <conditionalFormatting sqref="E462:F465">
+    <cfRule type="cellIs" dxfId="17" priority="23" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F464:F467">
-    <cfRule type="cellIs" dxfId="21" priority="21" operator="equal">
+  <conditionalFormatting sqref="F462:F465">
+    <cfRule type="cellIs" dxfId="16" priority="21" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="22" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E468:F480">
-    <cfRule type="cellIs" dxfId="19" priority="19" operator="equal">
+  <conditionalFormatting sqref="E466:F478">
+    <cfRule type="cellIs" dxfId="14" priority="19" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="20" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E468:F480">
-    <cfRule type="cellIs" dxfId="17" priority="18" operator="equal">
+  <conditionalFormatting sqref="E466:F478">
+    <cfRule type="cellIs" dxfId="12" priority="18" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F468:F480">
-    <cfRule type="cellIs" dxfId="16" priority="16" operator="equal">
+  <conditionalFormatting sqref="F466:F478">
+    <cfRule type="cellIs" dxfId="11" priority="16" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="17" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E484:F485">
-    <cfRule type="cellIs" dxfId="14" priority="14" operator="equal">
+  <conditionalFormatting sqref="E482:F483">
+    <cfRule type="cellIs" dxfId="9" priority="14" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="15" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E484:F485">
-    <cfRule type="cellIs" dxfId="12" priority="13" operator="equal">
+  <conditionalFormatting sqref="E482:F483">
+    <cfRule type="cellIs" dxfId="7" priority="13" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F484:F485">
-    <cfRule type="cellIs" dxfId="11" priority="11" operator="equal">
+  <conditionalFormatting sqref="F482:F483">
+    <cfRule type="cellIs" dxfId="6" priority="11" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="12" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E486:F488">
-    <cfRule type="cellIs" dxfId="9" priority="9" operator="equal">
+  <conditionalFormatting sqref="E484:F486">
+    <cfRule type="cellIs" dxfId="4" priority="9" operator="equal">
       <formula>"ex"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="10" operator="equal">
       <formula>"in"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E486:F488">
-    <cfRule type="cellIs" dxfId="7" priority="8" operator="equal">
+  <conditionalFormatting sqref="E484:F486">
+    <cfRule type="cellIs" dxfId="2" priority="8" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F486:F488">
-    <cfRule type="cellIs" dxfId="6" priority="6" operator="equal">
+  <conditionalFormatting sqref="F484:F486">
+    <cfRule type="cellIs" dxfId="1" priority="6" operator="equal">
       <formula>"ft"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
-      <formula>"seg"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E489:F489">
-    <cfRule type="cellIs" dxfId="4" priority="4" operator="equal">
-      <formula>"ex"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="5" operator="equal">
-      <formula>"in"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E489:F489">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
-      <formula>"ft"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F489">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
-      <formula>"ft"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="7" operator="equal">
       <formula>"seg"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>